<commit_message>
(v3.0.1.9059) Update taxonomy of microorganisms
</commit_message>
<xml_diff>
--- a/data-raw/datasets/microorganisms.groups.xlsx
+++ b/data-raw/datasets/microorganisms.groups.xlsx
@@ -369,8 +369,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:D535"/>
-  <sheetFormatPr baseColWidth="8.43" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:D531"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="e">
@@ -6976,7 +6976,7 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>B_HMPHL_QNTN</t>
+          <t>B_AGGRG_SGNS</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -6986,7 +6986,7 @@
       </c>
       <c r="D301" t="inlineStr">
         <is>
-          <t>Haemophilus quentini</t>
+          <t>Haemophilus segnis</t>
         </is>
       </c>
     </row>
@@ -6998,7 +6998,7 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>B_AGGRG_SGNS</t>
+          <t>B_HMPHL_SMNL</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -7008,7 +7008,7 @@
       </c>
       <c r="D302" t="inlineStr">
         <is>
-          <t>Haemophilus segnis</t>
+          <t>Haemophilus seminalis</t>
         </is>
       </c>
     </row>
@@ -7020,7 +7020,7 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>B_HMPHL_SMNL</t>
+          <t>B_HMPHL_SPTR</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
@@ -7030,7 +7030,7 @@
       </c>
       <c r="D303" t="inlineStr">
         <is>
-          <t>Haemophilus seminalis</t>
+          <t>Haemophilus sputorum</t>
         </is>
       </c>
     </row>
@@ -7042,7 +7042,7 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>B_HMPHL_SPTR</t>
+          <t>B_GRDNR_VGNL</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -7052,7 +7052,7 @@
       </c>
       <c r="D304" t="inlineStr">
         <is>
-          <t>Haemophilus sputorum</t>
+          <t>Haemophilus vaginalis</t>
         </is>
       </c>
     </row>
@@ -7064,7 +7064,7 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>B_GRDNR_VGNL</t>
+          <t>B_KGLLA</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -7074,7 +7074,7 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Haemophilus vaginalis</t>
+          <t>Kingella</t>
         </is>
       </c>
     </row>
@@ -7086,7 +7086,7 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>B_KGLLA</t>
+          <t>B_KGLLA_DNTR</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -7096,7 +7096,7 @@
       </c>
       <c r="D306" t="inlineStr">
         <is>
-          <t>Kingella</t>
+          <t>Kingella denitrificans</t>
         </is>
       </c>
     </row>
@@ -7108,7 +7108,7 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>B_KGLLA_DNTR</t>
+          <t>B_STTNL_INDL</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
@@ -7118,7 +7118,7 @@
       </c>
       <c r="D307" t="inlineStr">
         <is>
-          <t>Kingella denitrificans</t>
+          <t>Kingella indologenes</t>
         </is>
       </c>
     </row>
@@ -7130,7 +7130,7 @@
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>B_STTNL_INDL</t>
+          <t>B_KGLLA_KING</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -7140,7 +7140,7 @@
       </c>
       <c r="D308" t="inlineStr">
         <is>
-          <t>Kingella indologenes</t>
+          <t>Kingella kingae</t>
         </is>
       </c>
     </row>
@@ -7152,7 +7152,7 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>B_KGLLA_KING</t>
+          <t>B_KGLLA_NGVN</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -7162,7 +7162,7 @@
       </c>
       <c r="D309" t="inlineStr">
         <is>
-          <t>Kingella kingae</t>
+          <t>Kingella negevensis</t>
         </is>
       </c>
     </row>
@@ -7174,7 +7174,7 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>B_KGLLA_NGVN</t>
+          <t>B_KGLLA_ORLS</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="D310" t="inlineStr">
         <is>
-          <t>Kingella negevensis</t>
+          <t>Kingella orale</t>
         </is>
       </c>
     </row>
@@ -7206,7 +7206,7 @@
       </c>
       <c r="D311" t="inlineStr">
         <is>
-          <t>Kingella orale</t>
+          <t>Kingella oralis</t>
         </is>
       </c>
     </row>
@@ -7218,7 +7218,7 @@
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>B_KGLLA_ORLS</t>
+          <t>B_KGLLA_POTS</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
@@ -7228,29 +7228,29 @@
       </c>
       <c r="D312" t="inlineStr">
         <is>
-          <t>Kingella oralis</t>
+          <t>Kingella potus</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>B_HACEK</t>
+          <t>B_KLBSL_PNMN-C</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>B_KGLLA_POTS</t>
+          <t>B_KLBSL_AFRC</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>Haemophilus, Aggregatibacter, Cardiobacterium, Eikenella, Kingella (HACEK)</t>
+          <t>Klebsiella pneumoniae complex</t>
         </is>
       </c>
       <c r="D313" t="inlineStr">
         <is>
-          <t>Kingella potus</t>
+          <t>Klebsiella africana</t>
         </is>
       </c>
     </row>
@@ -7262,7 +7262,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>B_KLBSL_AFRC</t>
+          <t>B_KLBSL_PNMN</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -7272,7 +7272,7 @@
       </c>
       <c r="D314" t="inlineStr">
         <is>
-          <t>Klebsiella africana</t>
+          <t>Klebsiella pneumoniae</t>
         </is>
       </c>
     </row>
@@ -7284,7 +7284,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>B_KLBSL_PNMN</t>
+          <t>B_KLBSL_PNMN_OZAN</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -7294,7 +7294,7 @@
       </c>
       <c r="D315" t="inlineStr">
         <is>
-          <t>Klebsiella pneumoniae</t>
+          <t>Klebsiella pneumoniae ozaenae</t>
         </is>
       </c>
     </row>
@@ -7306,7 +7306,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>B_KLBSL_PNMN_OZAN</t>
+          <t>B_KLBSL_PNMN_PNMN</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -7316,7 +7316,7 @@
       </c>
       <c r="D316" t="inlineStr">
         <is>
-          <t>Klebsiella pneumoniae ozaenae</t>
+          <t>Klebsiella pneumoniae pneumoniae</t>
         </is>
       </c>
     </row>
@@ -7328,7 +7328,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>B_KLBSL_PNMN_PNMN</t>
+          <t>B_KLBSL_PNMN_RHNS</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -7338,7 +7338,7 @@
       </c>
       <c r="D317" t="inlineStr">
         <is>
-          <t>Klebsiella pneumoniae pneumoniae</t>
+          <t>Klebsiella pneumoniae rhinoscleromatis</t>
         </is>
       </c>
     </row>
@@ -7350,7 +7350,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>B_KLBSL_PNMN_RHNS</t>
+          <t>B_KLBSL_QSPN</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -7360,7 +7360,7 @@
       </c>
       <c r="D318" t="inlineStr">
         <is>
-          <t>Klebsiella pneumoniae rhinoscleromatis</t>
+          <t>Klebsiella quasipneumoniae</t>
         </is>
       </c>
     </row>
@@ -7372,7 +7372,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>B_KLBSL_QSPN</t>
+          <t>B_KLBSL_QSPN_QSPN</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -7382,7 +7382,7 @@
       </c>
       <c r="D319" t="inlineStr">
         <is>
-          <t>Klebsiella quasipneumoniae</t>
+          <t>Klebsiella quasipneumoniae quasipneumoniae</t>
         </is>
       </c>
     </row>
@@ -7394,7 +7394,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>B_KLBSL_QSPN_QSPN</t>
+          <t>B_KLBSL_QSPN_SMLP</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -7404,7 +7404,7 @@
       </c>
       <c r="D320" t="inlineStr">
         <is>
-          <t>Klebsiella quasipneumoniae quasipneumoniae</t>
+          <t>Klebsiella quasipneumoniae similipneumoniae</t>
         </is>
       </c>
     </row>
@@ -7416,7 +7416,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>B_KLBSL_QSPN_SMLP</t>
+          <t>B_KLBSL_VRCL</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -7426,7 +7426,7 @@
       </c>
       <c r="D321" t="inlineStr">
         <is>
-          <t>Klebsiella quasipneumoniae similipneumoniae</t>
+          <t>Klebsiella variicola</t>
         </is>
       </c>
     </row>
@@ -7438,7 +7438,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>B_KLBSL_QSVR</t>
+          <t>B_KLBSL_VRCL_TRPC</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -7448,7 +7448,7 @@
       </c>
       <c r="D322" t="inlineStr">
         <is>
-          <t>Klebsiella quasivariicola</t>
+          <t>Klebsiella variicola tropica</t>
         </is>
       </c>
     </row>
@@ -7460,7 +7460,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>B_KLBSL_VRCL</t>
+          <t>B_KLBSL_VRCL_LNSS</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -7470,7 +7470,7 @@
       </c>
       <c r="D323" t="inlineStr">
         <is>
-          <t>Klebsiella variicola</t>
+          <t>Klebsiella variicola tropicalensis</t>
         </is>
       </c>
     </row>
@@ -7482,7 +7482,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>B_KLBSL_VRCL_TRPC</t>
+          <t>B_KLBSL_VRCL_VRCL</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -7492,51 +7492,51 @@
       </c>
       <c r="D324" t="inlineStr">
         <is>
-          <t>Klebsiella variicola tropica</t>
+          <t>Klebsiella variicola variicola</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>B_KLBSL_PNMN-C</t>
+          <t>F_MYRZY_GLLR-C</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>B_KLBSL_VRCL_LNSS</t>
+          <t>F_CANDD_FRMN</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>Klebsiella pneumoniae complex</t>
+          <t>Meyerozyma guilliermondii complex</t>
         </is>
       </c>
       <c r="D325" t="inlineStr">
         <is>
-          <t>Klebsiella variicola tropicalensis</t>
+          <t>Candida fermentati</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>B_KLBSL_PNMN-C</t>
+          <t>F_MYRZY_GLLR-C</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>B_KLBSL_VRCL_VRCL</t>
+          <t>F_MYRZY_CRBB</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>Klebsiella pneumoniae complex</t>
+          <t>Meyerozyma guilliermondii complex</t>
         </is>
       </c>
       <c r="D326" t="inlineStr">
         <is>
-          <t>Klebsiella variicola variicola</t>
+          <t>Meyerozyma caribbica</t>
         </is>
       </c>
     </row>
@@ -7548,7 +7548,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>F_CANDD_FRMN</t>
+          <t>F_MYRZY_CRPP</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -7558,7 +7558,7 @@
       </c>
       <c r="D327" t="inlineStr">
         <is>
-          <t>Candida fermentati</t>
+          <t>Meyerozyma carpophila</t>
         </is>
       </c>
     </row>
@@ -7570,7 +7570,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>F_MYRZY_CRBB</t>
+          <t>F_MYRZY_GLLR</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -7580,7 +7580,7 @@
       </c>
       <c r="D328" t="inlineStr">
         <is>
-          <t>Meyerozyma caribbica</t>
+          <t>Meyerozyma guilliermondii</t>
         </is>
       </c>
     </row>
@@ -7602,7 +7602,7 @@
       </c>
       <c r="D329" t="inlineStr">
         <is>
-          <t>Meyerozyma carpophila</t>
+          <t>Meyerozyma guilliermondii carpophila</t>
         </is>
       </c>
     </row>
@@ -7624,7 +7624,7 @@
       </c>
       <c r="D330" t="inlineStr">
         <is>
-          <t>Meyerozyma guilliermondii</t>
+          <t>Meyerozyma guilliermondii japonica</t>
         </is>
       </c>
     </row>
@@ -7636,7 +7636,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>F_MYRZY_CRPP</t>
+          <t>F_MYRZY_GLLR</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -7646,7 +7646,7 @@
       </c>
       <c r="D331" t="inlineStr">
         <is>
-          <t>Meyerozyma guilliermondii carpophila</t>
+          <t>Meyerozyma guilliermondii muhira</t>
         </is>
       </c>
     </row>
@@ -7668,51 +7668,51 @@
       </c>
       <c r="D332" t="inlineStr">
         <is>
-          <t>Meyerozyma guilliermondii japonica</t>
+          <t>Meyerozyma guilliermondii pseudoguilliermondii</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>F_MYRZY_GLLR-C</t>
+          <t>B_MYCBC_AVIM-C</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>F_MYRZY_GLLR</t>
+          <t>B_MYCBC_AVIM</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>Meyerozyma guilliermondii complex</t>
+          <t>Mycobacterium avium complex</t>
         </is>
       </c>
       <c r="D333" t="inlineStr">
         <is>
-          <t>Meyerozyma guilliermondii muhira</t>
+          <t>Mycobacterium avium</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>F_MYRZY_GLLR-C</t>
+          <t>B_MYCBC_AVIM-C</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>F_MYRZY_GLLR</t>
+          <t>B_MYCBC_AVIM_AVIM</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>Meyerozyma guilliermondii complex</t>
+          <t>Mycobacterium avium complex</t>
         </is>
       </c>
       <c r="D334" t="inlineStr">
         <is>
-          <t>Meyerozyma guilliermondii pseudoguilliermondii</t>
+          <t>Mycobacterium avium avium</t>
         </is>
       </c>
     </row>
@@ -7724,17 +7724,17 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>B_MYCBC_AVIM</t>
+          <t>B_MYCBC_AVIM_PRTB</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>Mycobacterium avium-intracellulare complex</t>
+          <t>Mycobacterium avium complex</t>
         </is>
       </c>
       <c r="D335" t="inlineStr">
         <is>
-          <t>Mycobacterium avium</t>
+          <t>Mycobacterium avium paratuberculosis</t>
         </is>
       </c>
     </row>
@@ -7746,17 +7746,17 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>B_MYCBC_AVIM_AVIM</t>
+          <t>B_MYCBC_AVIM_SLVT</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>Mycobacterium avium-intracellulare complex</t>
+          <t>Mycobacterium avium complex</t>
         </is>
       </c>
       <c r="D336" t="inlineStr">
         <is>
-          <t>Mycobacterium avium avium</t>
+          <t>Mycobacterium avium silvaticum</t>
         </is>
       </c>
     </row>
@@ -7768,17 +7768,17 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>B_MYCBC_AVIM_PRTB</t>
+          <t>B_MYCBC_LLRE</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>Mycobacterium avium-intracellulare complex</t>
+          <t>Mycobacterium avium complex</t>
         </is>
       </c>
       <c r="D337" t="inlineStr">
         <is>
-          <t>Mycobacterium avium paratuberculosis</t>
+          <t>Mycobacterium intracellulare</t>
         </is>
       </c>
     </row>
@@ -7790,17 +7790,17 @@
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>B_MYCBC_AVIM_SLVT</t>
+          <t>B_MYCBC_LLRE_CHMR</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>Mycobacterium avium-intracellulare complex</t>
+          <t>Mycobacterium avium complex</t>
         </is>
       </c>
       <c r="D338" t="inlineStr">
         <is>
-          <t>Mycobacterium avium silvaticum</t>
+          <t>Mycobacterium intracellulare chimaera</t>
         </is>
       </c>
     </row>
@@ -7812,17 +7812,17 @@
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>B_MYCBC_LLRE</t>
+          <t>B_MYCBC_LLRE_INTR</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>Mycobacterium avium-intracellulare complex</t>
+          <t>Mycobacterium avium complex</t>
         </is>
       </c>
       <c r="D339" t="inlineStr">
         <is>
-          <t>Mycobacterium intracellulare</t>
+          <t>Mycobacterium intracellulare intracellulare</t>
         </is>
       </c>
     </row>
@@ -7839,56 +7839,56 @@
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>Mycobacterium avium-intracellulare complex</t>
+          <t>Mycobacterium avium complex</t>
         </is>
       </c>
       <c r="D340" t="inlineStr">
         <is>
-          <t>Mycobacterium intracellulare chimaera</t>
+          <t>Mycobacterium intracellulare yongonense</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>B_MYCBC_AVIM-C</t>
+          <t>B_MYCBC_TBRC-C</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>B_MYCBC_LLRE_INTR</t>
+          <t>B_MYCBC_TBRC</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>Mycobacterium avium-intracellulare complex</t>
+          <t>Mycobacterium tuberculosis complex</t>
         </is>
       </c>
       <c r="D341" t="inlineStr">
         <is>
-          <t>Mycobacterium intracellulare intracellulare</t>
+          <t>Mycobacterium africanum</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>B_MYCBC_AVIM-C</t>
+          <t>B_MYCBC_TBRC-C</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>B_MYCBC_LLRE_CHMR</t>
+          <t>B_MYCBC_TBRC</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>Mycobacterium avium-intracellulare complex</t>
+          <t>Mycobacterium tuberculosis complex</t>
         </is>
       </c>
       <c r="D342" t="inlineStr">
         <is>
-          <t>Mycobacterium intracellulare yongonense</t>
+          <t>Mycobacterium bovis</t>
         </is>
       </c>
     </row>
@@ -7910,7 +7910,7 @@
       </c>
       <c r="D343" t="inlineStr">
         <is>
-          <t>Mycobacterium africanum</t>
+          <t>Mycobacterium bovis bovis</t>
         </is>
       </c>
     </row>
@@ -7932,7 +7932,7 @@
       </c>
       <c r="D344" t="inlineStr">
         <is>
-          <t>Mycobacterium bovis</t>
+          <t>Mycobacterium bovis caprae</t>
         </is>
       </c>
     </row>
@@ -7954,7 +7954,7 @@
       </c>
       <c r="D345" t="inlineStr">
         <is>
-          <t>Mycobacterium bovis bovis</t>
+          <t>Mycobacterium caprae</t>
         </is>
       </c>
     </row>
@@ -7976,7 +7976,7 @@
       </c>
       <c r="D346" t="inlineStr">
         <is>
-          <t>Mycobacterium bovis caprae</t>
+          <t>Mycobacterium microti</t>
         </is>
       </c>
     </row>
@@ -7998,7 +7998,7 @@
       </c>
       <c r="D347" t="inlineStr">
         <is>
-          <t>Mycobacterium caprae</t>
+          <t>Mycobacterium pinnipedii</t>
         </is>
       </c>
     </row>
@@ -8020,7 +8020,7 @@
       </c>
       <c r="D348" t="inlineStr">
         <is>
-          <t>Mycobacterium microti</t>
+          <t>Mycobacterium tuberculosis</t>
         </is>
       </c>
     </row>
@@ -8032,7 +8032,7 @@
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>B_MYCBC_MUNG</t>
+          <t>B_MYCBC_TBRC</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
@@ -8042,7 +8042,7 @@
       </c>
       <c r="D349" t="inlineStr">
         <is>
-          <t>Mycobacterium mungi</t>
+          <t>Mycobacterium tuberculosis caprae</t>
         </is>
       </c>
     </row>
@@ -8054,7 +8054,7 @@
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>B_MYCBC_ORYG</t>
+          <t>B_MYCBC_TBRC</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
@@ -8064,117 +8064,117 @@
       </c>
       <c r="D350" t="inlineStr">
         <is>
-          <t>Mycobacterium orygis</t>
+          <t>Mycobacterium tuberculosis tuberculosis</t>
         </is>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>B_MYCBC_TBRC-C</t>
+          <t>B_PSDMN_FLRS-C</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>B_MYCBC_TBRC</t>
+          <t>B_PSDMN_FLRS</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>Mycobacterium tuberculosis complex</t>
+          <t>Pseudomonas fluorescens complex</t>
         </is>
       </c>
       <c r="D351" t="inlineStr">
         <is>
-          <t>Mycobacterium pinnipedii</t>
+          <t>Pseudomonas fluorescens</t>
         </is>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>B_MYCBC_TBRC-C</t>
+          <t>B_MYCBC_RGM</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>B_MYCBC_TBRC</t>
+          <t>B_MYCBC_ABSC_ABSC</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>Mycobacterium tuberculosis complex</t>
+          <t>Rapidly growing Mycobacterium (RGM)</t>
         </is>
       </c>
       <c r="D352" t="inlineStr">
         <is>
-          <t>Mycobacterium tuberculosis</t>
+          <t>Mycobacterium abscessus abscessus</t>
         </is>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>B_MYCBC_TBRC-C</t>
+          <t>B_MYCBC_RGM</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>B_MYCBC_TBRC</t>
+          <t>B_MYCBC_ABSC_BLLT</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>Mycobacterium tuberculosis complex</t>
+          <t>Rapidly growing Mycobacterium (RGM)</t>
         </is>
       </c>
       <c r="D353" t="inlineStr">
         <is>
-          <t>Mycobacterium tuberculosis caprae</t>
+          <t>Mycobacterium abscessus bolletii</t>
         </is>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>B_MYCBC_TBRC-C</t>
+          <t>B_MYCBC_RGM</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>B_MYCBC_TBRC</t>
+          <t>B_MYCBC_ABSC_MSSL</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>Mycobacterium tuberculosis complex</t>
+          <t>Rapidly growing Mycobacterium (RGM)</t>
         </is>
       </c>
       <c r="D354" t="inlineStr">
         <is>
-          <t>Mycobacterium tuberculosis tuberculosis</t>
+          <t>Mycobacterium abscessus massiliense</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>B_PSDMN_FLRS-C</t>
+          <t>B_MYCBC_RGM</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>B_PSDMN_FLRS</t>
+          <t>B_MYCBC_AGRI</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>Pseudomonas fluorescens complex</t>
+          <t>Rapidly growing Mycobacterium (RGM)</t>
         </is>
       </c>
       <c r="D355" t="inlineStr">
         <is>
-          <t>Pseudomonas fluorescens</t>
+          <t>Mycobacterium agri</t>
         </is>
       </c>
     </row>
@@ -8186,7 +8186,7 @@
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>B_MYCBC_ABSC_ABSC</t>
+          <t>B_MYCBC_ACHN</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
@@ -8196,7 +8196,7 @@
       </c>
       <c r="D356" t="inlineStr">
         <is>
-          <t>Mycobacterium abscessus abscessus</t>
+          <t>Mycobacterium aichiense</t>
         </is>
       </c>
     </row>
@@ -8208,7 +8208,7 @@
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>B_MYCBC_ABSC_BLLT</t>
+          <t>B_MYCBC_ALGR</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
@@ -8218,7 +8218,7 @@
       </c>
       <c r="D357" t="inlineStr">
         <is>
-          <t>Mycobacterium abscessus bolletii</t>
+          <t>Mycobacterium algericum</t>
         </is>
       </c>
     </row>
@@ -8230,7 +8230,7 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>B_MYCBC_ABSC_MSSL</t>
+          <t>B_MYCBC_ALVE</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
@@ -8240,7 +8240,7 @@
       </c>
       <c r="D358" t="inlineStr">
         <is>
-          <t>Mycobacterium abscessus massiliense</t>
+          <t>Mycobacterium alvei</t>
         </is>
       </c>
     </row>
@@ -8252,7 +8252,7 @@
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>B_MYCBC_AGRI</t>
+          <t>B_MYCBC_ANYN</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
@@ -8262,7 +8262,7 @@
       </c>
       <c r="D359" t="inlineStr">
         <is>
-          <t>Mycobacterium agri</t>
+          <t>Mycobacterium anyangense</t>
         </is>
       </c>
     </row>
@@ -8274,7 +8274,7 @@
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>B_MYCBC_ACHN</t>
+          <t>B_MYCBC_ARBN</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
@@ -8284,7 +8284,7 @@
       </c>
       <c r="D360" t="inlineStr">
         <is>
-          <t>Mycobacterium aichiense</t>
+          <t>Mycobacterium arabiense</t>
         </is>
       </c>
     </row>
@@ -8296,7 +8296,7 @@
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>B_MYCBC_ALGR</t>
+          <t>B_MYCBC_ARMT</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
@@ -8306,7 +8306,7 @@
       </c>
       <c r="D361" t="inlineStr">
         <is>
-          <t>Mycobacterium algericum</t>
+          <t>Mycobacterium aromaticivorans</t>
         </is>
       </c>
     </row>
@@ -8318,7 +8318,7 @@
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>B_MYCBC_ALVE</t>
+          <t>B_MYCBC_ABGN</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
@@ -8328,7 +8328,7 @@
       </c>
       <c r="D362" t="inlineStr">
         <is>
-          <t>Mycobacterium alvei</t>
+          <t>Mycobacterium aubagnense</t>
         </is>
       </c>
     </row>
@@ -8340,7 +8340,7 @@
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>B_MYCBC_ANYN</t>
+          <t>B_MYCBC_AURM</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
@@ -8350,7 +8350,7 @@
       </c>
       <c r="D363" t="inlineStr">
         <is>
-          <t>Mycobacterium anyangense</t>
+          <t>Mycobacterium aurum</t>
         </is>
       </c>
     </row>
@@ -8362,7 +8362,7 @@
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>B_MYCBC_ARBN</t>
+          <t>B_MYCBC_ASTR</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
@@ -8372,7 +8372,7 @@
       </c>
       <c r="D364" t="inlineStr">
         <is>
-          <t>Mycobacterium arabiense</t>
+          <t>Mycobacterium austroafricanum</t>
         </is>
       </c>
     </row>
@@ -8384,7 +8384,7 @@
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>B_MYCBC_ARMT</t>
+          <t>B_MYCBC_BCTR</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
@@ -8394,7 +8394,7 @@
       </c>
       <c r="D365" t="inlineStr">
         <is>
-          <t>Mycobacterium aromaticivorans</t>
+          <t>Mycobacterium bacteremicum</t>
         </is>
       </c>
     </row>
@@ -8406,7 +8406,7 @@
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>B_MYCBC_ABGN</t>
+          <t>B_MYCBC_BNCK</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
@@ -8416,7 +8416,7 @@
       </c>
       <c r="D366" t="inlineStr">
         <is>
-          <t>Mycobacterium aubagnense</t>
+          <t>Mycobacterium boenickei</t>
         </is>
       </c>
     </row>
@@ -8428,7 +8428,7 @@
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>B_MYCBC_AURM</t>
+          <t>B_MYCBC_BRGL</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
@@ -8438,7 +8438,7 @@
       </c>
       <c r="D367" t="inlineStr">
         <is>
-          <t>Mycobacterium aurum</t>
+          <t>Mycobacterium bourgelatii</t>
         </is>
       </c>
     </row>
@@ -8450,7 +8450,7 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>B_MYCBC_ASTR</t>
+          <t>B_MYCBC_BRSB</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
@@ -8460,7 +8460,7 @@
       </c>
       <c r="D368" t="inlineStr">
         <is>
-          <t>Mycobacterium austroafricanum</t>
+          <t>Mycobacterium brisbanense</t>
         </is>
       </c>
     </row>
@@ -8472,7 +8472,7 @@
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>B_MYCBC_BCTR</t>
+          <t>B_MYCBC_BRUM</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
@@ -8482,7 +8482,7 @@
       </c>
       <c r="D369" t="inlineStr">
         <is>
-          <t>Mycobacterium bacteremicum</t>
+          <t>Mycobacterium brumae</t>
         </is>
       </c>
     </row>
@@ -8494,7 +8494,7 @@
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>B_MYCBC_BNCK</t>
+          <t>B_MYCBC_CNRS</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
@@ -8504,7 +8504,7 @@
       </c>
       <c r="D370" t="inlineStr">
         <is>
-          <t>Mycobacterium boenickei</t>
+          <t>Mycobacterium canariasense</t>
         </is>
       </c>
     </row>
@@ -8516,7 +8516,7 @@
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t>B_MYCBC_BRGL</t>
+          <t>B_MYCBC_CLRF</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
@@ -8526,7 +8526,7 @@
       </c>
       <c r="D371" t="inlineStr">
         <is>
-          <t>Mycobacterium bourgelatii</t>
+          <t>Mycobacterium celeriflavum</t>
         </is>
       </c>
     </row>
@@ -8538,7 +8538,7 @@
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t>B_MYCBC_BRSB</t>
+          <t>B_MYCBC_CHLN</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
@@ -8548,7 +8548,7 @@
       </c>
       <c r="D372" t="inlineStr">
         <is>
-          <t>Mycobacterium brisbanense</t>
+          <t>Mycobacterium chelonae</t>
         </is>
       </c>
     </row>
@@ -8560,7 +8560,7 @@
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t>B_MYCBC_BRUM</t>
+          <t>B_MYCBC_ABSC</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
@@ -8570,7 +8570,7 @@
       </c>
       <c r="D373" t="inlineStr">
         <is>
-          <t>Mycobacterium brumae</t>
+          <t>Mycobacterium chelonae abscessus</t>
         </is>
       </c>
     </row>
@@ -8582,7 +8582,7 @@
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t>B_MYCBC_CNRS</t>
+          <t>B_MYCBC_CHLN_BVST</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
@@ -8592,7 +8592,7 @@
       </c>
       <c r="D374" t="inlineStr">
         <is>
-          <t>Mycobacterium canariasense</t>
+          <t>Mycobacterium chelonae bovis</t>
         </is>
       </c>
     </row>
@@ -8604,7 +8604,7 @@
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t>B_MYCBC_CLRF</t>
+          <t>B_MYCBC_CHLN_CHLN</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
@@ -8614,7 +8614,7 @@
       </c>
       <c r="D375" t="inlineStr">
         <is>
-          <t>Mycobacterium celeriflavum</t>
+          <t>Mycobacterium chelonae chelonae</t>
         </is>
       </c>
     </row>
@@ -8626,7 +8626,7 @@
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t>B_MYCBC_CHLN</t>
+          <t>B_MYCBC_CHLN_GWNK</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
@@ -8636,7 +8636,7 @@
       </c>
       <c r="D376" t="inlineStr">
         <is>
-          <t>Mycobacterium chelonae</t>
+          <t>Mycobacterium chelonae gwanakae</t>
         </is>
       </c>
     </row>
@@ -8648,7 +8648,7 @@
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t>B_MYCBC_ABSC</t>
+          <t>B_MYCBC_CHIT</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
@@ -8658,7 +8658,7 @@
       </c>
       <c r="D377" t="inlineStr">
         <is>
-          <t>Mycobacterium chelonae abscessus</t>
+          <t>Mycobacterium chitae</t>
         </is>
       </c>
     </row>
@@ -8670,7 +8670,7 @@
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t>B_MYCBC_CHLN_BVST</t>
+          <t>B_MYCBC_CHLR</t>
         </is>
       </c>
       <c r="C378" t="inlineStr">
@@ -8680,7 +8680,7 @@
       </c>
       <c r="D378" t="inlineStr">
         <is>
-          <t>Mycobacterium chelonae bovis</t>
+          <t>Mycobacterium chlorophenolicum</t>
         </is>
       </c>
     </row>
@@ -8692,7 +8692,7 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t>B_MYCBC_CHLN_CHLN</t>
+          <t>B_MYCBC_CHBN</t>
         </is>
       </c>
       <c r="C379" t="inlineStr">
@@ -8702,7 +8702,7 @@
       </c>
       <c r="D379" t="inlineStr">
         <is>
-          <t>Mycobacterium chelonae chelonae</t>
+          <t>Mycobacterium chubuense</t>
         </is>
       </c>
     </row>
@@ -8714,7 +8714,7 @@
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>B_MYCBC_CHLN_GWNK</t>
+          <t>B_MYCBC_CNFL</t>
         </is>
       </c>
       <c r="C380" t="inlineStr">
@@ -8724,7 +8724,7 @@
       </c>
       <c r="D380" t="inlineStr">
         <is>
-          <t>Mycobacterium chelonae gwanakae</t>
+          <t>Mycobacterium confluentis</t>
         </is>
       </c>
     </row>
@@ -8736,7 +8736,7 @@
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t>B_MYCBC_CHIT</t>
+          <t>B_MYCBC_CSMT</t>
         </is>
       </c>
       <c r="C381" t="inlineStr">
@@ -8746,7 +8746,7 @@
       </c>
       <c r="D381" t="inlineStr">
         <is>
-          <t>Mycobacterium chitae</t>
+          <t>Mycobacterium cosmeticum</t>
         </is>
       </c>
     </row>
@@ -8758,7 +8758,7 @@
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t>B_MYCBC_CHLR</t>
+          <t>B_MYCBC_CRCN</t>
         </is>
       </c>
       <c r="C382" t="inlineStr">
@@ -8768,7 +8768,7 @@
       </c>
       <c r="D382" t="inlineStr">
         <is>
-          <t>Mycobacterium chlorophenolicum</t>
+          <t>Mycobacterium crocinum</t>
         </is>
       </c>
     </row>
@@ -8780,7 +8780,7 @@
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t>B_MYCBC_CHBN</t>
+          <t>B_MYCBC_DRNH</t>
         </is>
       </c>
       <c r="C383" t="inlineStr">
@@ -8790,7 +8790,7 @@
       </c>
       <c r="D383" t="inlineStr">
         <is>
-          <t>Mycobacterium chubuense</t>
+          <t>Mycobacterium diernhoferi</t>
         </is>
       </c>
     </row>
@@ -8802,7 +8802,7 @@
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t>B_MYCBC_CNFL</t>
+          <t>B_MYCBC_DUVL</t>
         </is>
       </c>
       <c r="C384" t="inlineStr">
@@ -8812,7 +8812,7 @@
       </c>
       <c r="D384" t="inlineStr">
         <is>
-          <t>Mycobacterium confluentis</t>
+          <t>Mycobacterium duvalii</t>
         </is>
       </c>
     </row>
@@ -8824,7 +8824,7 @@
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t>B_MYCBC_CSMT</t>
+          <t>B_MYCBC_ELPH</t>
         </is>
       </c>
       <c r="C385" t="inlineStr">
@@ -8834,7 +8834,7 @@
       </c>
       <c r="D385" t="inlineStr">
         <is>
-          <t>Mycobacterium cosmeticum</t>
+          <t>Mycobacterium elephantis</t>
         </is>
       </c>
     </row>
@@ -8846,7 +8846,7 @@
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t>B_MYCBC_CRCN</t>
+          <t>B_MYCBC_FLLX</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
@@ -8856,7 +8856,7 @@
       </c>
       <c r="D386" t="inlineStr">
         <is>
-          <t>Mycobacterium crocinum</t>
+          <t>Mycobacterium fallax</t>
         </is>
       </c>
     </row>
@@ -8868,7 +8868,7 @@
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t>B_MYCBC_DRNH</t>
+          <t>B_MYCBC_FLVS</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
@@ -8878,7 +8878,7 @@
       </c>
       <c r="D387" t="inlineStr">
         <is>
-          <t>Mycobacterium diernhoferi</t>
+          <t>Mycobacterium flavescens</t>
         </is>
       </c>
     </row>
@@ -8890,7 +8890,7 @@
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t>B_MYCBC_DUVL</t>
+          <t>B_MYCBC_VRNS</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
@@ -8900,7 +8900,7 @@
       </c>
       <c r="D388" t="inlineStr">
         <is>
-          <t>Mycobacterium duvalii</t>
+          <t>Mycobacterium fluoranthenivorans</t>
         </is>
       </c>
     </row>
@@ -8912,7 +8912,7 @@
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t>B_MYCBC_ELPH</t>
+          <t>B_MYCBC_FRTT</t>
         </is>
       </c>
       <c r="C389" t="inlineStr">
@@ -8922,7 +8922,7 @@
       </c>
       <c r="D389" t="inlineStr">
         <is>
-          <t>Mycobacterium elephantis</t>
+          <t>Mycobacterium fortuitum</t>
         </is>
       </c>
     </row>
@@ -8934,7 +8934,7 @@
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t>B_MYCBC_FLLX</t>
+          <t>B_MYCBC_FRTT_ACTM</t>
         </is>
       </c>
       <c r="C390" t="inlineStr">
@@ -8944,7 +8944,7 @@
       </c>
       <c r="D390" t="inlineStr">
         <is>
-          <t>Mycobacterium fallax</t>
+          <t>Mycobacterium fortuitum acetamidolyticum</t>
         </is>
       </c>
     </row>
@@ -8956,7 +8956,7 @@
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t>B_MYCBC_FLVS</t>
+          <t>B_MYCBC_FRTT_FRTT</t>
         </is>
       </c>
       <c r="C391" t="inlineStr">
@@ -8966,7 +8966,7 @@
       </c>
       <c r="D391" t="inlineStr">
         <is>
-          <t>Mycobacterium flavescens</t>
+          <t>Mycobacterium fortuitum fortuitum</t>
         </is>
       </c>
     </row>
@@ -8978,7 +8978,7 @@
       </c>
       <c r="B392" t="inlineStr">
         <is>
-          <t>B_MYCBC_VRNS</t>
+          <t>B_MYCBC_FRNK</t>
         </is>
       </c>
       <c r="C392" t="inlineStr">
@@ -8988,7 +8988,7 @@
       </c>
       <c r="D392" t="inlineStr">
         <is>
-          <t>Mycobacterium fluoranthenivorans</t>
+          <t>Mycobacterium franklinii</t>
         </is>
       </c>
     </row>
@@ -9000,7 +9000,7 @@
       </c>
       <c r="B393" t="inlineStr">
         <is>
-          <t>B_MYCBC_FRTT</t>
+          <t>B_MYCBC_FRDR</t>
         </is>
       </c>
       <c r="C393" t="inlineStr">
@@ -9010,7 +9010,7 @@
       </c>
       <c r="D393" t="inlineStr">
         <is>
-          <t>Mycobacterium fortuitum</t>
+          <t>Mycobacterium frederiksbergense</t>
         </is>
       </c>
     </row>
@@ -9022,7 +9022,7 @@
       </c>
       <c r="B394" t="inlineStr">
         <is>
-          <t>B_MYCBC_FRTT_ACTM</t>
+          <t>B_MYCBC_GADM</t>
         </is>
       </c>
       <c r="C394" t="inlineStr">
@@ -9032,7 +9032,7 @@
       </c>
       <c r="D394" t="inlineStr">
         <is>
-          <t>Mycobacterium fortuitum acetamidolyticum</t>
+          <t>Mycobacterium gadium</t>
         </is>
       </c>
     </row>
@@ -9044,7 +9044,7 @@
       </c>
       <c r="B395" t="inlineStr">
         <is>
-          <t>B_MYCBC_FRTT_FRTT</t>
+          <t>B_MYCBC_GLVM</t>
         </is>
       </c>
       <c r="C395" t="inlineStr">
@@ -9054,7 +9054,7 @@
       </c>
       <c r="D395" t="inlineStr">
         <is>
-          <t>Mycobacterium fortuitum fortuitum</t>
+          <t>Mycobacterium gilvum</t>
         </is>
       </c>
     </row>
@@ -9066,7 +9066,7 @@
       </c>
       <c r="B396" t="inlineStr">
         <is>
-          <t>B_MYCBC_FRNK</t>
+          <t>B_MYCBC_GOOD</t>
         </is>
       </c>
       <c r="C396" t="inlineStr">
@@ -9076,7 +9076,7 @@
       </c>
       <c r="D396" t="inlineStr">
         <is>
-          <t>Mycobacterium franklinii</t>
+          <t>Mycobacterium goodii</t>
         </is>
       </c>
     </row>
@@ -9088,7 +9088,7 @@
       </c>
       <c r="B397" t="inlineStr">
         <is>
-          <t>B_MYCBC_FRDR</t>
+          <t>B_MYCBC_HSSC</t>
         </is>
       </c>
       <c r="C397" t="inlineStr">
@@ -9098,7 +9098,7 @@
       </c>
       <c r="D397" t="inlineStr">
         <is>
-          <t>Mycobacterium frederiksbergense</t>
+          <t>Mycobacterium hassiacum</t>
         </is>
       </c>
     </row>
@@ -9110,7 +9110,7 @@
       </c>
       <c r="B398" t="inlineStr">
         <is>
-          <t>B_MYCBC_GADM</t>
+          <t>B_MYCBC_HPPC</t>
         </is>
       </c>
       <c r="C398" t="inlineStr">
@@ -9120,7 +9120,7 @@
       </c>
       <c r="D398" t="inlineStr">
         <is>
-          <t>Mycobacterium gadium</t>
+          <t>Mycobacterium hippocampi</t>
         </is>
       </c>
     </row>
@@ -9132,7 +9132,7 @@
       </c>
       <c r="B399" t="inlineStr">
         <is>
-          <t>B_MYCBC_GLVM</t>
+          <t>B_MYCBC_HDLR</t>
         </is>
       </c>
       <c r="C399" t="inlineStr">
@@ -9142,7 +9142,7 @@
       </c>
       <c r="D399" t="inlineStr">
         <is>
-          <t>Mycobacterium gilvum</t>
+          <t>Mycobacterium hodleri</t>
         </is>
       </c>
     </row>
@@ -9154,7 +9154,7 @@
       </c>
       <c r="B400" t="inlineStr">
         <is>
-          <t>B_MYCBC_GOOD</t>
+          <t>B_MYCBC_HLST</t>
         </is>
       </c>
       <c r="C400" t="inlineStr">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="D400" t="inlineStr">
         <is>
-          <t>Mycobacterium goodii</t>
+          <t>Mycobacterium holsaticum</t>
         </is>
       </c>
     </row>
@@ -9176,7 +9176,7 @@
       </c>
       <c r="B401" t="inlineStr">
         <is>
-          <t>B_MYCBC_HSSC</t>
+          <t>B_MYCBC_HSTN</t>
         </is>
       </c>
       <c r="C401" t="inlineStr">
@@ -9186,7 +9186,7 @@
       </c>
       <c r="D401" t="inlineStr">
         <is>
-          <t>Mycobacterium hassiacum</t>
+          <t>Mycobacterium houstonense</t>
         </is>
       </c>
     </row>
@@ -9198,7 +9198,7 @@
       </c>
       <c r="B402" t="inlineStr">
         <is>
-          <t>B_MYCBC_HPPC</t>
+          <t>B_MYCBC_IMMN</t>
         </is>
       </c>
       <c r="C402" t="inlineStr">
@@ -9208,7 +9208,7 @@
       </c>
       <c r="D402" t="inlineStr">
         <is>
-          <t>Mycobacterium hippocampi</t>
+          <t>Mycobacterium immunogenum</t>
         </is>
       </c>
     </row>
@@ -9220,7 +9220,7 @@
       </c>
       <c r="B403" t="inlineStr">
         <is>
-          <t>B_MYCBC_HDLR</t>
+          <t>B_MYCBC_INSB</t>
         </is>
       </c>
       <c r="C403" t="inlineStr">
@@ -9230,7 +9230,7 @@
       </c>
       <c r="D403" t="inlineStr">
         <is>
-          <t>Mycobacterium hodleri</t>
+          <t>Mycobacterium insubricum</t>
         </is>
       </c>
     </row>
@@ -9242,7 +9242,7 @@
       </c>
       <c r="B404" t="inlineStr">
         <is>
-          <t>B_MYCBC_HLST</t>
+          <t>B_MYCBC_IRNC</t>
         </is>
       </c>
       <c r="C404" t="inlineStr">
@@ -9252,7 +9252,7 @@
       </c>
       <c r="D404" t="inlineStr">
         <is>
-          <t>Mycobacterium holsaticum</t>
+          <t>Mycobacterium iranicum</t>
         </is>
       </c>
     </row>
@@ -9264,7 +9264,7 @@
       </c>
       <c r="B405" t="inlineStr">
         <is>
-          <t>B_MYCBC_HSTN</t>
+          <t>B_MYCBC_KMSS</t>
         </is>
       </c>
       <c r="C405" t="inlineStr">
@@ -9274,7 +9274,7 @@
       </c>
       <c r="D405" t="inlineStr">
         <is>
-          <t>Mycobacterium houstonense</t>
+          <t>Mycobacterium komossense</t>
         </is>
       </c>
     </row>
@@ -9286,7 +9286,7 @@
       </c>
       <c r="B406" t="inlineStr">
         <is>
-          <t>B_MYCBC_IMMN</t>
+          <t>B_MYCBC_LTRL</t>
         </is>
       </c>
       <c r="C406" t="inlineStr">
@@ -9296,7 +9296,7 @@
       </c>
       <c r="D406" t="inlineStr">
         <is>
-          <t>Mycobacterium immunogenum</t>
+          <t>Mycobacterium litorale</t>
         </is>
       </c>
     </row>
@@ -9308,7 +9308,7 @@
       </c>
       <c r="B407" t="inlineStr">
         <is>
-          <t>B_MYCBC_INSB</t>
+          <t>B_MYCBC_LLTZ</t>
         </is>
       </c>
       <c r="C407" t="inlineStr">
@@ -9318,7 +9318,7 @@
       </c>
       <c r="D407" t="inlineStr">
         <is>
-          <t>Mycobacterium insubricum</t>
+          <t>Mycobacterium llatzerense</t>
         </is>
       </c>
     </row>
@@ -9330,7 +9330,7 @@
       </c>
       <c r="B408" t="inlineStr">
         <is>
-          <t>B_MYCBC_IRNC</t>
+          <t>B_MYCBC_MDGS</t>
         </is>
       </c>
       <c r="C408" t="inlineStr">
@@ -9340,7 +9340,7 @@
       </c>
       <c r="D408" t="inlineStr">
         <is>
-          <t>Mycobacterium iranicum</t>
+          <t>Mycobacterium madagascariense</t>
         </is>
       </c>
     </row>
@@ -9352,7 +9352,7 @@
       </c>
       <c r="B409" t="inlineStr">
         <is>
-          <t>B_MYCBC_KMSS</t>
+          <t>B_MYCBC_MGRT</t>
         </is>
       </c>
       <c r="C409" t="inlineStr">
@@ -9362,7 +9362,7 @@
       </c>
       <c r="D409" t="inlineStr">
         <is>
-          <t>Mycobacterium komossense</t>
+          <t>Mycobacterium mageritense</t>
         </is>
       </c>
     </row>
@@ -9374,7 +9374,7 @@
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>B_MYCBC_LTRL</t>
+          <t>B_MYCBC_MNCN</t>
         </is>
       </c>
       <c r="C410" t="inlineStr">
@@ -9384,7 +9384,7 @@
       </c>
       <c r="D410" t="inlineStr">
         <is>
-          <t>Mycobacterium litorale</t>
+          <t>Mycobacterium monacense</t>
         </is>
       </c>
     </row>
@@ -9396,7 +9396,7 @@
       </c>
       <c r="B411" t="inlineStr">
         <is>
-          <t>B_MYCBC_LLTZ</t>
+          <t>B_MYCBC_MRKN</t>
         </is>
       </c>
       <c r="C411" t="inlineStr">
@@ -9406,7 +9406,7 @@
       </c>
       <c r="D411" t="inlineStr">
         <is>
-          <t>Mycobacterium llatzerense</t>
+          <t>Mycobacterium moriokaense</t>
         </is>
       </c>
     </row>
@@ -9418,7 +9418,7 @@
       </c>
       <c r="B412" t="inlineStr">
         <is>
-          <t>B_MYCBC_MDGS</t>
+          <t>B_MYCBC_MCGN</t>
         </is>
       </c>
       <c r="C412" t="inlineStr">
@@ -9428,7 +9428,7 @@
       </c>
       <c r="D412" t="inlineStr">
         <is>
-          <t>Mycobacterium madagascariense</t>
+          <t>Mycobacterium mucogenicum</t>
         </is>
       </c>
     </row>
@@ -9440,7 +9440,7 @@
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>B_MYCBC_MGRT</t>
+          <t>B_MYCBC_MURL</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
@@ -9450,7 +9450,7 @@
       </c>
       <c r="D413" t="inlineStr">
         <is>
-          <t>Mycobacterium mageritense</t>
+          <t>Mycobacterium murale</t>
         </is>
       </c>
     </row>
@@ -9462,7 +9462,7 @@
       </c>
       <c r="B414" t="inlineStr">
         <is>
-          <t>B_MYCBC_MNCN</t>
+          <t>B_MYCBC_NERM</t>
         </is>
       </c>
       <c r="C414" t="inlineStr">
@@ -9472,7 +9472,7 @@
       </c>
       <c r="D414" t="inlineStr">
         <is>
-          <t>Mycobacterium monacense</t>
+          <t>Mycobacterium neoaurum</t>
         </is>
       </c>
     </row>
@@ -9484,7 +9484,7 @@
       </c>
       <c r="B415" t="inlineStr">
         <is>
-          <t>B_MYCBC_MRKN</t>
+          <t>B_MYCBC_NWRL</t>
         </is>
       </c>
       <c r="C415" t="inlineStr">
@@ -9494,7 +9494,7 @@
       </c>
       <c r="D415" t="inlineStr">
         <is>
-          <t>Mycobacterium moriokaense</t>
+          <t>Mycobacterium neworleansense</t>
         </is>
       </c>
     </row>
@@ -9506,7 +9506,7 @@
       </c>
       <c r="B416" t="inlineStr">
         <is>
-          <t>B_MYCBC_MCGN</t>
+          <t>B_MYCBC_NVCS</t>
         </is>
       </c>
       <c r="C416" t="inlineStr">
@@ -9516,7 +9516,7 @@
       </c>
       <c r="D416" t="inlineStr">
         <is>
-          <t>Mycobacterium mucogenicum</t>
+          <t>Mycobacterium novocastrense</t>
         </is>
       </c>
     </row>
@@ -9528,7 +9528,7 @@
       </c>
       <c r="B417" t="inlineStr">
         <is>
-          <t>B_MYCBC_MURL</t>
+          <t>B_MYCBC_OBNS</t>
         </is>
       </c>
       <c r="C417" t="inlineStr">
@@ -9538,7 +9538,7 @@
       </c>
       <c r="D417" t="inlineStr">
         <is>
-          <t>Mycobacterium murale</t>
+          <t>Mycobacterium obuense</t>
         </is>
       </c>
     </row>
@@ -9550,7 +9550,7 @@
       </c>
       <c r="B418" t="inlineStr">
         <is>
-          <t>B_MYCBC_NERM</t>
+          <t>B_MYCBC_PLLN</t>
         </is>
       </c>
       <c r="C418" t="inlineStr">
@@ -9560,7 +9560,7 @@
       </c>
       <c r="D418" t="inlineStr">
         <is>
-          <t>Mycobacterium neoaurum</t>
+          <t>Mycobacterium pallens</t>
         </is>
       </c>
     </row>
@@ -9572,7 +9572,7 @@
       </c>
       <c r="B419" t="inlineStr">
         <is>
-          <t>B_MYCBC_NWRL</t>
+          <t>B_MYCBC_PRFR</t>
         </is>
       </c>
       <c r="C419" t="inlineStr">
@@ -9582,7 +9582,7 @@
       </c>
       <c r="D419" t="inlineStr">
         <is>
-          <t>Mycobacterium neworleansense</t>
+          <t>Mycobacterium parafortuitum</t>
         </is>
       </c>
     </row>
@@ -9594,7 +9594,7 @@
       </c>
       <c r="B420" t="inlineStr">
         <is>
-          <t>B_MYCBC_NVCS</t>
+          <t>B_MYCBC_GRNM</t>
         </is>
       </c>
       <c r="C420" t="inlineStr">
@@ -9604,7 +9604,7 @@
       </c>
       <c r="D420" t="inlineStr">
         <is>
-          <t>Mycobacterium novocastrense</t>
+          <t>Mycobacterium peregrinum</t>
         </is>
       </c>
     </row>
@@ -9616,7 +9616,7 @@
       </c>
       <c r="B421" t="inlineStr">
         <is>
-          <t>B_MYCBC_OBNS</t>
+          <t>B_MYCBC_PHLE</t>
         </is>
       </c>
       <c r="C421" t="inlineStr">
@@ -9626,7 +9626,7 @@
       </c>
       <c r="D421" t="inlineStr">
         <is>
-          <t>Mycobacterium obuense</t>
+          <t>Mycobacterium phlei</t>
         </is>
       </c>
     </row>
@@ -9638,7 +9638,7 @@
       </c>
       <c r="B422" t="inlineStr">
         <is>
-          <t>B_MYCBC_PLLN</t>
+          <t>B_MYCBC_PHCC</t>
         </is>
       </c>
       <c r="C422" t="inlineStr">
@@ -9648,7 +9648,7 @@
       </c>
       <c r="D422" t="inlineStr">
         <is>
-          <t>Mycobacterium pallens</t>
+          <t>Mycobacterium phocaicum</t>
         </is>
       </c>
     </row>
@@ -9660,7 +9660,7 @@
       </c>
       <c r="B423" t="inlineStr">
         <is>
-          <t>B_MYCBC_PRFR</t>
+          <t>B_MYCBC_PRCN</t>
         </is>
       </c>
       <c r="C423" t="inlineStr">
@@ -9670,7 +9670,7 @@
       </c>
       <c r="D423" t="inlineStr">
         <is>
-          <t>Mycobacterium parafortuitum</t>
+          <t>Mycobacterium porcinum</t>
         </is>
       </c>
     </row>
@@ -9682,7 +9682,7 @@
       </c>
       <c r="B424" t="inlineStr">
         <is>
-          <t>B_MYCBC_GRNM</t>
+          <t>B_MYCBC_RFRE</t>
         </is>
       </c>
       <c r="C424" t="inlineStr">
@@ -9692,7 +9692,7 @@
       </c>
       <c r="D424" t="inlineStr">
         <is>
-          <t>Mycobacterium peregrinum</t>
+          <t>Mycobacterium poriferae</t>
         </is>
       </c>
     </row>
@@ -9704,7 +9704,7 @@
       </c>
       <c r="B425" t="inlineStr">
         <is>
-          <t>B_MYCBC_PHLE</t>
+          <t>B_MYCBC_PSYC</t>
         </is>
       </c>
       <c r="C425" t="inlineStr">
@@ -9714,7 +9714,7 @@
       </c>
       <c r="D425" t="inlineStr">
         <is>
-          <t>Mycobacterium phlei</t>
+          <t>Mycobacterium psychrotolerans</t>
         </is>
       </c>
     </row>
@@ -9726,7 +9726,7 @@
       </c>
       <c r="B426" t="inlineStr">
         <is>
-          <t>B_MYCBC_PHCC</t>
+          <t>B_MYCBC_PYRN</t>
         </is>
       </c>
       <c r="C426" t="inlineStr">
@@ -9736,7 +9736,7 @@
       </c>
       <c r="D426" t="inlineStr">
         <is>
-          <t>Mycobacterium phocaicum</t>
+          <t>Mycobacterium pyrenivorans</t>
         </is>
       </c>
     </row>
@@ -9748,7 +9748,7 @@
       </c>
       <c r="B427" t="inlineStr">
         <is>
-          <t>B_MYCBC_PRCN</t>
+          <t>B_MYCBC_RHDS</t>
         </is>
       </c>
       <c r="C427" t="inlineStr">
@@ -9758,7 +9758,7 @@
       </c>
       <c r="D427" t="inlineStr">
         <is>
-          <t>Mycobacterium porcinum</t>
+          <t>Mycobacterium rhodesiae</t>
         </is>
       </c>
     </row>
@@ -9770,7 +9770,7 @@
       </c>
       <c r="B428" t="inlineStr">
         <is>
-          <t>B_MYCBC_RFRE</t>
+          <t>B_MYCBC_RUFM</t>
         </is>
       </c>
       <c r="C428" t="inlineStr">
@@ -9780,7 +9780,7 @@
       </c>
       <c r="D428" t="inlineStr">
         <is>
-          <t>Mycobacterium poriferae</t>
+          <t>Mycobacterium rufum</t>
         </is>
       </c>
     </row>
@@ -9792,7 +9792,7 @@
       </c>
       <c r="B429" t="inlineStr">
         <is>
-          <t>B_MYCBC_PSYC</t>
+          <t>B_MYCBC_RTLM</t>
         </is>
       </c>
       <c r="C429" t="inlineStr">
@@ -9802,7 +9802,7 @@
       </c>
       <c r="D429" t="inlineStr">
         <is>
-          <t>Mycobacterium psychrotolerans</t>
+          <t>Mycobacterium rutilum</t>
         </is>
       </c>
     </row>
@@ -9814,7 +9814,7 @@
       </c>
       <c r="B430" t="inlineStr">
         <is>
-          <t>B_MYCBC_PYRN</t>
+          <t>B_MYCBC_SLMN</t>
         </is>
       </c>
       <c r="C430" t="inlineStr">
@@ -9824,7 +9824,7 @@
       </c>
       <c r="D430" t="inlineStr">
         <is>
-          <t>Mycobacterium pyrenivorans</t>
+          <t>Mycobacterium salmoniphilum</t>
         </is>
       </c>
     </row>
@@ -9836,7 +9836,7 @@
       </c>
       <c r="B431" t="inlineStr">
         <is>
-          <t>B_MYCBC_RHDS</t>
+          <t>B_MYCBC_SDMN</t>
         </is>
       </c>
       <c r="C431" t="inlineStr">
@@ -9846,7 +9846,7 @@
       </c>
       <c r="D431" t="inlineStr">
         <is>
-          <t>Mycobacterium rhodesiae</t>
+          <t>Mycobacterium sediminis</t>
         </is>
       </c>
     </row>
@@ -9858,7 +9858,7 @@
       </c>
       <c r="B432" t="inlineStr">
         <is>
-          <t>B_MYCBC_RUFM</t>
+          <t>B_MYCBC_SNGL</t>
         </is>
       </c>
       <c r="C432" t="inlineStr">
@@ -9868,7 +9868,7 @@
       </c>
       <c r="D432" t="inlineStr">
         <is>
-          <t>Mycobacterium rufum</t>
+          <t>Mycobacterium senegalense</t>
         </is>
       </c>
     </row>
@@ -9880,7 +9880,7 @@
       </c>
       <c r="B433" t="inlineStr">
         <is>
-          <t>B_MYCBC_RTLM</t>
+          <t>B_MYCBC_SPTC</t>
         </is>
       </c>
       <c r="C433" t="inlineStr">
@@ -9890,7 +9890,7 @@
       </c>
       <c r="D433" t="inlineStr">
         <is>
-          <t>Mycobacterium rutilum</t>
+          <t>Mycobacterium septicum</t>
         </is>
       </c>
     </row>
@@ -9902,7 +9902,7 @@
       </c>
       <c r="B434" t="inlineStr">
         <is>
-          <t>B_MYCBC_SLMN</t>
+          <t>B_MYCBC_STNS</t>
         </is>
       </c>
       <c r="C434" t="inlineStr">
@@ -9912,7 +9912,7 @@
       </c>
       <c r="D434" t="inlineStr">
         <is>
-          <t>Mycobacterium salmoniphilum</t>
+          <t>Mycobacterium setense</t>
         </is>
       </c>
     </row>
@@ -9924,7 +9924,7 @@
       </c>
       <c r="B435" t="inlineStr">
         <is>
-          <t>B_MYCBC_SDMN</t>
+          <t>B_MYCBC_SMGM</t>
         </is>
       </c>
       <c r="C435" t="inlineStr">
@@ -9934,7 +9934,7 @@
       </c>
       <c r="D435" t="inlineStr">
         <is>
-          <t>Mycobacterium sediminis</t>
+          <t>Mycobacterium smegmatis</t>
         </is>
       </c>
     </row>
@@ -9946,7 +9946,7 @@
       </c>
       <c r="B436" t="inlineStr">
         <is>
-          <t>B_MYCBC_SNGL</t>
+          <t>B_MYCBC_SPHG</t>
         </is>
       </c>
       <c r="C436" t="inlineStr">
@@ -9956,7 +9956,7 @@
       </c>
       <c r="D436" t="inlineStr">
         <is>
-          <t>Mycobacterium senegalense</t>
+          <t>Mycobacterium sphagni</t>
         </is>
       </c>
     </row>
@@ -9968,7 +9968,7 @@
       </c>
       <c r="B437" t="inlineStr">
         <is>
-          <t>B_MYCBC_SPTC</t>
+          <t>B_MYCBC_THRM</t>
         </is>
       </c>
       <c r="C437" t="inlineStr">
@@ -9978,7 +9978,7 @@
       </c>
       <c r="D437" t="inlineStr">
         <is>
-          <t>Mycobacterium septicum</t>
+          <t>Mycobacterium thermoresistibile</t>
         </is>
       </c>
     </row>
@@ -9990,7 +9990,7 @@
       </c>
       <c r="B438" t="inlineStr">
         <is>
-          <t>B_MYCBC_STNS</t>
+          <t>B_MYCBC_TKNS</t>
         </is>
       </c>
       <c r="C438" t="inlineStr">
@@ -10000,7 +10000,7 @@
       </c>
       <c r="D438" t="inlineStr">
         <is>
-          <t>Mycobacterium setense</t>
+          <t>Mycobacterium tokaiense</t>
         </is>
       </c>
     </row>
@@ -10012,7 +10012,7 @@
       </c>
       <c r="B439" t="inlineStr">
         <is>
-          <t>B_MYCBC_SMGM</t>
+          <t>B_MYCBC_VACC</t>
         </is>
       </c>
       <c r="C439" t="inlineStr">
@@ -10022,7 +10022,7 @@
       </c>
       <c r="D439" t="inlineStr">
         <is>
-          <t>Mycobacterium smegmatis</t>
+          <t>Mycobacterium vaccae</t>
         </is>
       </c>
     </row>
@@ -10034,7 +10034,7 @@
       </c>
       <c r="B440" t="inlineStr">
         <is>
-          <t>B_MYCBC_SPHG</t>
+          <t>B_MYCBC_ASTR</t>
         </is>
       </c>
       <c r="C440" t="inlineStr">
@@ -10044,7 +10044,7 @@
       </c>
       <c r="D440" t="inlineStr">
         <is>
-          <t>Mycobacterium sphagni</t>
+          <t>Mycobacterium vanbaalenii</t>
         </is>
       </c>
     </row>
@@ -10056,7 +10056,7 @@
       </c>
       <c r="B441" t="inlineStr">
         <is>
-          <t>B_MYCBC_THRM</t>
+          <t>B_MYCBC_WLNS</t>
         </is>
       </c>
       <c r="C441" t="inlineStr">
@@ -10066,95 +10066,95 @@
       </c>
       <c r="D441" t="inlineStr">
         <is>
-          <t>Mycobacterium thermoresistibile</t>
+          <t>Mycobacterium wolinskyi</t>
         </is>
       </c>
     </row>
     <row r="442">
       <c r="A442" t="inlineStr">
         <is>
-          <t>B_MYCBC_RGM</t>
+          <t>B_MYCBC_SGM</t>
         </is>
       </c>
       <c r="B442" t="inlineStr">
         <is>
-          <t>B_MYCBC_TKNS</t>
+          <t>B_MYCBC_FRCN</t>
         </is>
       </c>
       <c r="C442" t="inlineStr">
         <is>
-          <t>Rapidly growing Mycobacterium (RGM)</t>
+          <t>Slowly growing Mycobacterium (SGM)</t>
         </is>
       </c>
       <c r="D442" t="inlineStr">
         <is>
-          <t>Mycobacterium tokaiense</t>
+          <t>Mycobacterium farcinogenes</t>
         </is>
       </c>
     </row>
     <row r="443">
       <c r="A443" t="inlineStr">
         <is>
-          <t>B_MYCBC_RGM</t>
+          <t>B_MYCBC_SGM</t>
         </is>
       </c>
       <c r="B443" t="inlineStr">
         <is>
-          <t>B_MYCBC_VACC</t>
+          <t>B_MYCBC_GSTR</t>
         </is>
       </c>
       <c r="C443" t="inlineStr">
         <is>
-          <t>Rapidly growing Mycobacterium (RGM)</t>
+          <t>Slowly growing Mycobacterium (SGM)</t>
         </is>
       </c>
       <c r="D443" t="inlineStr">
         <is>
-          <t>Mycobacterium vaccae</t>
+          <t>Mycobacterium gastri</t>
         </is>
       </c>
     </row>
     <row r="444">
       <c r="A444" t="inlineStr">
         <is>
-          <t>B_MYCBC_RGM</t>
+          <t>B_MYCBC_SGM</t>
         </is>
       </c>
       <c r="B444" t="inlineStr">
         <is>
-          <t>B_MYCBC_ASTR</t>
+          <t>B_MYCBC_GNVN</t>
         </is>
       </c>
       <c r="C444" t="inlineStr">
         <is>
-          <t>Rapidly growing Mycobacterium (RGM)</t>
+          <t>Slowly growing Mycobacterium (SGM)</t>
         </is>
       </c>
       <c r="D444" t="inlineStr">
         <is>
-          <t>Mycobacterium vanbaalenii</t>
+          <t>Mycobacterium genavense</t>
         </is>
       </c>
     </row>
     <row r="445">
       <c r="A445" t="inlineStr">
         <is>
-          <t>B_MYCBC_RGM</t>
+          <t>B_MYCBC_SGM</t>
         </is>
       </c>
       <c r="B445" t="inlineStr">
         <is>
-          <t>B_MYCBC_WLNS</t>
+          <t>B_MYCBC_HMPH</t>
         </is>
       </c>
       <c r="C445" t="inlineStr">
         <is>
-          <t>Rapidly growing Mycobacterium (RGM)</t>
+          <t>Slowly growing Mycobacterium (SGM)</t>
         </is>
       </c>
       <c r="D445" t="inlineStr">
         <is>
-          <t>Mycobacterium wolinskyi</t>
+          <t>Mycobacterium haemophilum</t>
         </is>
       </c>
     </row>
@@ -10166,7 +10166,7 @@
       </c>
       <c r="B446" t="inlineStr">
         <is>
-          <t>B_MYCBC_FRCN</t>
+          <t>B_MYCBC_KNSS</t>
         </is>
       </c>
       <c r="C446" t="inlineStr">
@@ -10176,7 +10176,7 @@
       </c>
       <c r="D446" t="inlineStr">
         <is>
-          <t>Mycobacterium farcinogenes</t>
+          <t>Mycobacterium kansasii</t>
         </is>
       </c>
     </row>
@@ -10188,7 +10188,7 @@
       </c>
       <c r="B447" t="inlineStr">
         <is>
-          <t>B_MYCBC_GSTR</t>
+          <t>B_MYCBC_LEPR</t>
         </is>
       </c>
       <c r="C447" t="inlineStr">
@@ -10198,7 +10198,7 @@
       </c>
       <c r="D447" t="inlineStr">
         <is>
-          <t>Mycobacterium gastri</t>
+          <t>Mycobacterium leprae</t>
         </is>
       </c>
     </row>
@@ -10210,7 +10210,7 @@
       </c>
       <c r="B448" t="inlineStr">
         <is>
-          <t>B_MYCBC_GNVN</t>
+          <t>B_MYCBC_LPRM</t>
         </is>
       </c>
       <c r="C448" t="inlineStr">
@@ -10220,7 +10220,7 @@
       </c>
       <c r="D448" t="inlineStr">
         <is>
-          <t>Mycobacterium genavense</t>
+          <t>Mycobacterium lepraemurium</t>
         </is>
       </c>
     </row>
@@ -10232,7 +10232,7 @@
       </c>
       <c r="B449" t="inlineStr">
         <is>
-          <t>B_MYCBC_HMPH</t>
+          <t>B_MYCBC_MLMN</t>
         </is>
       </c>
       <c r="C449" t="inlineStr">
@@ -10242,7 +10242,7 @@
       </c>
       <c r="D449" t="inlineStr">
         <is>
-          <t>Mycobacterium haemophilum</t>
+          <t>Mycobacterium malmoense</t>
         </is>
       </c>
     </row>
@@ -10254,7 +10254,7 @@
       </c>
       <c r="B450" t="inlineStr">
         <is>
-          <t>B_MYCBC_KNSS</t>
+          <t>B_MYCBC_MRNM</t>
         </is>
       </c>
       <c r="C450" t="inlineStr">
@@ -10264,117 +10264,117 @@
       </c>
       <c r="D450" t="inlineStr">
         <is>
-          <t>Mycobacterium kansasii</t>
+          <t>Mycobacterium marinum</t>
         </is>
       </c>
     </row>
     <row r="451">
       <c r="A451" t="inlineStr">
         <is>
-          <t>B_MYCBC_SGM</t>
+          <t>B_STRPT_GRPA</t>
         </is>
       </c>
       <c r="B451" t="inlineStr">
         <is>
-          <t>B_MYCBC_LEPR</t>
+          <t>B_STRPT_PYGN</t>
         </is>
       </c>
       <c r="C451" t="inlineStr">
         <is>
-          <t>Slowly growing Mycobacterium (SGM)</t>
+          <t>Streptococcus Group A</t>
         </is>
       </c>
       <c r="D451" t="inlineStr">
         <is>
-          <t>Mycobacterium leprae</t>
+          <t>Streptococcus pyogenes</t>
         </is>
       </c>
     </row>
     <row r="452">
       <c r="A452" t="inlineStr">
         <is>
-          <t>B_MYCBC_SGM</t>
+          <t>B_STRPT_ABCG</t>
         </is>
       </c>
       <c r="B452" t="inlineStr">
         <is>
-          <t>B_MYCBC_LPRM</t>
+          <t>B_STRPT_GRPA</t>
         </is>
       </c>
       <c r="C452" t="inlineStr">
         <is>
-          <t>Slowly growing Mycobacterium (SGM)</t>
+          <t>Streptococcus Group A, B, C, G</t>
         </is>
       </c>
       <c r="D452" t="inlineStr">
         <is>
-          <t>Mycobacterium lepraemurium</t>
+          <t>Streptococcus Group A</t>
         </is>
       </c>
     </row>
     <row r="453">
       <c r="A453" t="inlineStr">
         <is>
-          <t>B_MYCBC_SGM</t>
+          <t>B_STRPT_ABCG</t>
         </is>
       </c>
       <c r="B453" t="inlineStr">
         <is>
-          <t>B_MYCBC_MLMN</t>
+          <t>B_STRPT_GRPB</t>
         </is>
       </c>
       <c r="C453" t="inlineStr">
         <is>
-          <t>Slowly growing Mycobacterium (SGM)</t>
+          <t>Streptococcus Group A, B, C, G</t>
         </is>
       </c>
       <c r="D453" t="inlineStr">
         <is>
-          <t>Mycobacterium malmoense</t>
+          <t>Streptococcus Group B</t>
         </is>
       </c>
     </row>
     <row r="454">
       <c r="A454" t="inlineStr">
         <is>
-          <t>B_MYCBC_SGM</t>
+          <t>B_STRPT_ABCG</t>
         </is>
       </c>
       <c r="B454" t="inlineStr">
         <is>
-          <t>B_MYCBC_MRNM</t>
+          <t>B_STRPT_GRPC</t>
         </is>
       </c>
       <c r="C454" t="inlineStr">
         <is>
-          <t>Slowly growing Mycobacterium (SGM)</t>
+          <t>Streptococcus Group A, B, C, G</t>
         </is>
       </c>
       <c r="D454" t="inlineStr">
         <is>
-          <t>Mycobacterium marinum</t>
+          <t>Streptococcus Group C</t>
         </is>
       </c>
     </row>
     <row r="455">
       <c r="A455" t="inlineStr">
         <is>
-          <t>B_STRPT_GRPA</t>
+          <t>B_STRPT_ABCG</t>
         </is>
       </c>
       <c r="B455" t="inlineStr">
         <is>
-          <t>B_STRPT_PYGN</t>
+          <t>B_STRPT_GRPG</t>
         </is>
       </c>
       <c r="C455" t="inlineStr">
         <is>
-          <t>Streptococcus Group A</t>
+          <t>Streptococcus Group A, B, C, G</t>
         </is>
       </c>
       <c r="D455" t="inlineStr">
         <is>
-          <t>Streptococcus pyogenes</t>
+          <t>Streptococcus Group G</t>
         </is>
       </c>
     </row>
@@ -10386,7 +10386,7 @@
       </c>
       <c r="B456" t="inlineStr">
         <is>
-          <t>B_STRPT_GRPA</t>
+          <t>B_STRPT_AGLC</t>
         </is>
       </c>
       <c r="C456" t="inlineStr">
@@ -10396,7 +10396,7 @@
       </c>
       <c r="D456" t="inlineStr">
         <is>
-          <t>Streptococcus Group A</t>
+          <t>Streptococcus agalactiae</t>
         </is>
       </c>
     </row>
@@ -10408,7 +10408,7 @@
       </c>
       <c r="B457" t="inlineStr">
         <is>
-          <t>B_STRPT_GRPB</t>
+          <t>B_STRPT_CANS</t>
         </is>
       </c>
       <c r="C457" t="inlineStr">
@@ -10418,7 +10418,7 @@
       </c>
       <c r="D457" t="inlineStr">
         <is>
-          <t>Streptococcus Group B</t>
+          <t>Streptococcus canis</t>
         </is>
       </c>
     </row>
@@ -10430,7 +10430,7 @@
       </c>
       <c r="B458" t="inlineStr">
         <is>
-          <t>B_STRPT_GRPC</t>
+          <t>B_STRPT_DYSG</t>
         </is>
       </c>
       <c r="C458" t="inlineStr">
@@ -10440,7 +10440,7 @@
       </c>
       <c r="D458" t="inlineStr">
         <is>
-          <t>Streptococcus Group C</t>
+          <t>Streptococcus dysgalactiae</t>
         </is>
       </c>
     </row>
@@ -10452,7 +10452,7 @@
       </c>
       <c r="B459" t="inlineStr">
         <is>
-          <t>B_STRPT_GRPG</t>
+          <t>B_STRPT_DYSG_DYSG</t>
         </is>
       </c>
       <c r="C459" t="inlineStr">
@@ -10462,7 +10462,7 @@
       </c>
       <c r="D459" t="inlineStr">
         <is>
-          <t>Streptococcus Group G</t>
+          <t>Streptococcus dysgalactiae dysgalactiae</t>
         </is>
       </c>
     </row>
@@ -10474,7 +10474,7 @@
       </c>
       <c r="B460" t="inlineStr">
         <is>
-          <t>B_STRPT_AGLC</t>
+          <t>B_STRPT_DYSG_EQSM</t>
         </is>
       </c>
       <c r="C460" t="inlineStr">
@@ -10484,7 +10484,7 @@
       </c>
       <c r="D460" t="inlineStr">
         <is>
-          <t>Streptococcus agalactiae</t>
+          <t>Streptococcus dysgalactiae equisimilis</t>
         </is>
       </c>
     </row>
@@ -10496,7 +10496,7 @@
       </c>
       <c r="B461" t="inlineStr">
         <is>
-          <t>B_STRPT_CANS</t>
+          <t>B_STRPT_EQUI</t>
         </is>
       </c>
       <c r="C461" t="inlineStr">
@@ -10506,7 +10506,7 @@
       </c>
       <c r="D461" t="inlineStr">
         <is>
-          <t>Streptococcus canis</t>
+          <t>Streptococcus equi</t>
         </is>
       </c>
     </row>
@@ -10518,7 +10518,7 @@
       </c>
       <c r="B462" t="inlineStr">
         <is>
-          <t>B_STRPT_DYSG</t>
+          <t>B_STRPT_EQUI_EQUI</t>
         </is>
       </c>
       <c r="C462" t="inlineStr">
@@ -10528,7 +10528,7 @@
       </c>
       <c r="D462" t="inlineStr">
         <is>
-          <t>Streptococcus dysgalactiae</t>
+          <t>Streptococcus equi equi</t>
         </is>
       </c>
     </row>
@@ -10540,7 +10540,7 @@
       </c>
       <c r="B463" t="inlineStr">
         <is>
-          <t>B_STRPT_DYSG_DYSG</t>
+          <t>B_STRPT_EQUI_RMNT</t>
         </is>
       </c>
       <c r="C463" t="inlineStr">
@@ -10550,7 +10550,7 @@
       </c>
       <c r="D463" t="inlineStr">
         <is>
-          <t>Streptococcus dysgalactiae dysgalactiae</t>
+          <t>Streptococcus equi ruminatorum</t>
         </is>
       </c>
     </row>
@@ -10562,7 +10562,7 @@
       </c>
       <c r="B464" t="inlineStr">
         <is>
-          <t>B_STRPT_DYSG_EQSM</t>
+          <t>B_STRPT_EQUI_ZPDM</t>
         </is>
       </c>
       <c r="C464" t="inlineStr">
@@ -10572,7 +10572,7 @@
       </c>
       <c r="D464" t="inlineStr">
         <is>
-          <t>Streptococcus dysgalactiae equisimilis</t>
+          <t>Streptococcus equi zooepidemicus</t>
         </is>
       </c>
     </row>
@@ -10584,7 +10584,7 @@
       </c>
       <c r="B465" t="inlineStr">
         <is>
-          <t>B_STRPT_EQUI</t>
+          <t>B_STRPT_PYGN</t>
         </is>
       </c>
       <c r="C465" t="inlineStr">
@@ -10594,117 +10594,117 @@
       </c>
       <c r="D465" t="inlineStr">
         <is>
-          <t>Streptococcus equi</t>
+          <t>Streptococcus pyogenes</t>
         </is>
       </c>
     </row>
     <row r="466">
       <c r="A466" t="inlineStr">
         <is>
-          <t>B_STRPT_ABCG</t>
+          <t>B_STRPT_GRPB</t>
         </is>
       </c>
       <c r="B466" t="inlineStr">
         <is>
-          <t>B_STRPT_EQUI_EQUI</t>
+          <t>B_STRPT_AGLC</t>
         </is>
       </c>
       <c r="C466" t="inlineStr">
         <is>
-          <t>Streptococcus Group A, B, C, G</t>
+          <t>Streptococcus Group B</t>
         </is>
       </c>
       <c r="D466" t="inlineStr">
         <is>
-          <t>Streptococcus equi equi</t>
+          <t>Streptococcus agalactiae</t>
         </is>
       </c>
     </row>
     <row r="467">
       <c r="A467" t="inlineStr">
         <is>
-          <t>B_STRPT_ABCG</t>
+          <t>B_STRPT_GRPC</t>
         </is>
       </c>
       <c r="B467" t="inlineStr">
         <is>
-          <t>B_STRPT_EQUI_RMNT</t>
+          <t>B_STRPT_DYSG</t>
         </is>
       </c>
       <c r="C467" t="inlineStr">
         <is>
-          <t>Streptococcus Group A, B, C, G</t>
+          <t>Streptococcus Group C</t>
         </is>
       </c>
       <c r="D467" t="inlineStr">
         <is>
-          <t>Streptococcus equi ruminatorum</t>
+          <t>Streptococcus dysgalactiae</t>
         </is>
       </c>
     </row>
     <row r="468">
       <c r="A468" t="inlineStr">
         <is>
-          <t>B_STRPT_ABCG</t>
+          <t>B_STRPT_GRPC</t>
         </is>
       </c>
       <c r="B468" t="inlineStr">
         <is>
-          <t>B_STRPT_EQUI_ZPDM</t>
+          <t>B_STRPT_DYSG_DYSG</t>
         </is>
       </c>
       <c r="C468" t="inlineStr">
         <is>
-          <t>Streptococcus Group A, B, C, G</t>
+          <t>Streptococcus Group C</t>
         </is>
       </c>
       <c r="D468" t="inlineStr">
         <is>
-          <t>Streptococcus equi zooepidemicus</t>
+          <t>Streptococcus dysgalactiae dysgalactiae</t>
         </is>
       </c>
     </row>
     <row r="469">
       <c r="A469" t="inlineStr">
         <is>
-          <t>B_STRPT_ABCG</t>
+          <t>B_STRPT_GRPC</t>
         </is>
       </c>
       <c r="B469" t="inlineStr">
         <is>
-          <t>B_STRPT_PYGN</t>
+          <t>B_STRPT_DYSG_EQSM</t>
         </is>
       </c>
       <c r="C469" t="inlineStr">
         <is>
-          <t>Streptococcus Group A, B, C, G</t>
+          <t>Streptococcus Group C</t>
         </is>
       </c>
       <c r="D469" t="inlineStr">
         <is>
-          <t>Streptococcus pyogenes</t>
+          <t>Streptococcus dysgalactiae equisimilis</t>
         </is>
       </c>
     </row>
     <row r="470">
       <c r="A470" t="inlineStr">
         <is>
-          <t>B_STRPT_GRPB</t>
+          <t>B_STRPT_GRPC</t>
         </is>
       </c>
       <c r="B470" t="inlineStr">
         <is>
-          <t>B_STRPT_AGLC</t>
+          <t>B_STRPT_EQUI</t>
         </is>
       </c>
       <c r="C470" t="inlineStr">
         <is>
-          <t>Streptococcus Group B</t>
+          <t>Streptococcus Group C</t>
         </is>
       </c>
       <c r="D470" t="inlineStr">
         <is>
-          <t>Streptococcus agalactiae</t>
+          <t>Streptococcus equi</t>
         </is>
       </c>
     </row>
@@ -10716,7 +10716,7 @@
       </c>
       <c r="B471" t="inlineStr">
         <is>
-          <t>B_STRPT_DYSG</t>
+          <t>B_STRPT_EQUI_EQUI</t>
         </is>
       </c>
       <c r="C471" t="inlineStr">
@@ -10726,7 +10726,7 @@
       </c>
       <c r="D471" t="inlineStr">
         <is>
-          <t>Streptococcus dysgalactiae</t>
+          <t>Streptococcus equi equi</t>
         </is>
       </c>
     </row>
@@ -10738,7 +10738,7 @@
       </c>
       <c r="B472" t="inlineStr">
         <is>
-          <t>B_STRPT_DYSG_DYSG</t>
+          <t>B_STRPT_EQUI_RMNT</t>
         </is>
       </c>
       <c r="C472" t="inlineStr">
@@ -10748,7 +10748,7 @@
       </c>
       <c r="D472" t="inlineStr">
         <is>
-          <t>Streptococcus dysgalactiae dysgalactiae</t>
+          <t>Streptococcus equi ruminatorum</t>
         </is>
       </c>
     </row>
@@ -10760,7 +10760,7 @@
       </c>
       <c r="B473" t="inlineStr">
         <is>
-          <t>B_STRPT_DYSG_EQSM</t>
+          <t>B_STRPT_EQUI_ZPDM</t>
         </is>
       </c>
       <c r="C473" t="inlineStr">
@@ -10770,95 +10770,95 @@
       </c>
       <c r="D473" t="inlineStr">
         <is>
-          <t>Streptococcus dysgalactiae equisimilis</t>
+          <t>Streptococcus equi zooepidemicus</t>
         </is>
       </c>
     </row>
     <row r="474">
       <c r="A474" t="inlineStr">
         <is>
-          <t>B_STRPT_GRPC</t>
+          <t>B_STRPT_GRPF</t>
         </is>
       </c>
       <c r="B474" t="inlineStr">
         <is>
-          <t>B_STRPT_EQUI</t>
+          <t>B_STRPT_ANGN</t>
         </is>
       </c>
       <c r="C474" t="inlineStr">
         <is>
-          <t>Streptococcus Group C</t>
+          <t>Streptococcus Group F</t>
         </is>
       </c>
       <c r="D474" t="inlineStr">
         <is>
-          <t>Streptococcus equi</t>
+          <t>Streptococcus anginosus</t>
         </is>
       </c>
     </row>
     <row r="475">
       <c r="A475" t="inlineStr">
         <is>
-          <t>B_STRPT_GRPC</t>
+          <t>B_STRPT_GRPF</t>
         </is>
       </c>
       <c r="B475" t="inlineStr">
         <is>
-          <t>B_STRPT_EQUI_EQUI</t>
+          <t>B_STRPT_ANGN_ANGN</t>
         </is>
       </c>
       <c r="C475" t="inlineStr">
         <is>
-          <t>Streptococcus Group C</t>
+          <t>Streptococcus Group F</t>
         </is>
       </c>
       <c r="D475" t="inlineStr">
         <is>
-          <t>Streptococcus equi equi</t>
+          <t>Streptococcus anginosus anginosus</t>
         </is>
       </c>
     </row>
     <row r="476">
       <c r="A476" t="inlineStr">
         <is>
-          <t>B_STRPT_GRPC</t>
+          <t>B_STRPT_GRPF</t>
         </is>
       </c>
       <c r="B476" t="inlineStr">
         <is>
-          <t>B_STRPT_EQUI_RMNT</t>
+          <t>B_STRPT_ANGN_WHLY</t>
         </is>
       </c>
       <c r="C476" t="inlineStr">
         <is>
-          <t>Streptococcus Group C</t>
+          <t>Streptococcus Group F</t>
         </is>
       </c>
       <c r="D476" t="inlineStr">
         <is>
-          <t>Streptococcus equi ruminatorum</t>
+          <t>Streptococcus anginosus whileyi</t>
         </is>
       </c>
     </row>
     <row r="477">
       <c r="A477" t="inlineStr">
         <is>
-          <t>B_STRPT_GRPC</t>
+          <t>B_STRPT_GRPF</t>
         </is>
       </c>
       <c r="B477" t="inlineStr">
         <is>
-          <t>B_STRPT_EQUI_ZPDM</t>
+          <t>B_STRPT_CNST</t>
         </is>
       </c>
       <c r="C477" t="inlineStr">
         <is>
-          <t>Streptococcus Group C</t>
+          <t>Streptococcus Group F</t>
         </is>
       </c>
       <c r="D477" t="inlineStr">
         <is>
-          <t>Streptococcus equi zooepidemicus</t>
+          <t>Streptococcus constellatus</t>
         </is>
       </c>
     </row>
@@ -10870,7 +10870,7 @@
       </c>
       <c r="B478" t="inlineStr">
         <is>
-          <t>B_STRPT_ANGN</t>
+          <t>B_STRPT_CNST_CNST</t>
         </is>
       </c>
       <c r="C478" t="inlineStr">
@@ -10880,7 +10880,7 @@
       </c>
       <c r="D478" t="inlineStr">
         <is>
-          <t>Streptococcus anginosus</t>
+          <t>Streptococcus constellatus constellatus</t>
         </is>
       </c>
     </row>
@@ -10892,7 +10892,7 @@
       </c>
       <c r="B479" t="inlineStr">
         <is>
-          <t>B_STRPT_ANGN_ANGN</t>
+          <t>B_STRPT_CNST_PHRY</t>
         </is>
       </c>
       <c r="C479" t="inlineStr">
@@ -10902,7 +10902,7 @@
       </c>
       <c r="D479" t="inlineStr">
         <is>
-          <t>Streptococcus anginosus anginosus</t>
+          <t>Streptococcus constellatus pharyngis</t>
         </is>
       </c>
     </row>
@@ -10914,7 +10914,7 @@
       </c>
       <c r="B480" t="inlineStr">
         <is>
-          <t>B_STRPT_ANGN_WHLY</t>
+          <t>B_STRPT_CNST_VBRG</t>
         </is>
       </c>
       <c r="C480" t="inlineStr">
@@ -10924,7 +10924,7 @@
       </c>
       <c r="D480" t="inlineStr">
         <is>
-          <t>Streptococcus anginosus whileyi</t>
+          <t>Streptococcus constellatus viborgensis</t>
         </is>
       </c>
     </row>
@@ -10936,7 +10936,7 @@
       </c>
       <c r="B481" t="inlineStr">
         <is>
-          <t>B_STRPT_CNST</t>
+          <t>B_STRPT_INTR</t>
         </is>
       </c>
       <c r="C481" t="inlineStr">
@@ -10946,337 +10946,337 @@
       </c>
       <c r="D481" t="inlineStr">
         <is>
-          <t>Streptococcus constellatus</t>
+          <t>Streptococcus intermedius</t>
         </is>
       </c>
     </row>
     <row r="482">
       <c r="A482" t="inlineStr">
         <is>
-          <t>B_STRPT_GRPF</t>
+          <t>B_STRPT_GRPG</t>
         </is>
       </c>
       <c r="B482" t="inlineStr">
         <is>
-          <t>B_STRPT_CNST_CNST</t>
+          <t>B_STRPT_CANS</t>
         </is>
       </c>
       <c r="C482" t="inlineStr">
         <is>
-          <t>Streptococcus Group F</t>
+          <t>Streptococcus Group G</t>
         </is>
       </c>
       <c r="D482" t="inlineStr">
         <is>
-          <t>Streptococcus constellatus constellatus</t>
+          <t>Streptococcus canis</t>
         </is>
       </c>
     </row>
     <row r="483">
       <c r="A483" t="inlineStr">
         <is>
-          <t>B_STRPT_GRPF</t>
+          <t>B_STRPT_GRPG</t>
         </is>
       </c>
       <c r="B483" t="inlineStr">
         <is>
-          <t>B_STRPT_CNST_PHRY</t>
+          <t>B_STRPT_DYSG</t>
         </is>
       </c>
       <c r="C483" t="inlineStr">
         <is>
-          <t>Streptococcus Group F</t>
+          <t>Streptococcus Group G</t>
         </is>
       </c>
       <c r="D483" t="inlineStr">
         <is>
-          <t>Streptococcus constellatus pharyngis</t>
+          <t>Streptococcus dysgalactiae</t>
         </is>
       </c>
     </row>
     <row r="484">
       <c r="A484" t="inlineStr">
         <is>
-          <t>B_STRPT_GRPF</t>
+          <t>B_STRPT_GRPG</t>
         </is>
       </c>
       <c r="B484" t="inlineStr">
         <is>
-          <t>B_STRPT_CNST_VBRG</t>
+          <t>B_STRPT_DYSG_DYSG</t>
         </is>
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t>Streptococcus Group F</t>
+          <t>Streptococcus Group G</t>
         </is>
       </c>
       <c r="D484" t="inlineStr">
         <is>
-          <t>Streptococcus constellatus viborgensis</t>
+          <t>Streptococcus dysgalactiae dysgalactiae</t>
         </is>
       </c>
     </row>
     <row r="485">
       <c r="A485" t="inlineStr">
         <is>
-          <t>B_STRPT_GRPF</t>
+          <t>B_STRPT_GRPG</t>
         </is>
       </c>
       <c r="B485" t="inlineStr">
         <is>
-          <t>B_STRPT_INTR</t>
+          <t>B_STRPT_DYSG_EQSM</t>
         </is>
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>Streptococcus Group F</t>
+          <t>Streptococcus Group G</t>
         </is>
       </c>
       <c r="D485" t="inlineStr">
         <is>
-          <t>Streptococcus intermedius</t>
+          <t>Streptococcus dysgalactiae equisimilis</t>
         </is>
       </c>
     </row>
     <row r="486">
       <c r="A486" t="inlineStr">
         <is>
-          <t>B_STRPT_GRPG</t>
+          <t>B_STRPT_GRPH</t>
         </is>
       </c>
       <c r="B486" t="inlineStr">
         <is>
-          <t>B_STRPT_CANS</t>
+          <t>B_STRPT_SNGN</t>
         </is>
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>Streptococcus Group G</t>
+          <t>Streptococcus Group H</t>
         </is>
       </c>
       <c r="D486" t="inlineStr">
         <is>
-          <t>Streptococcus canis</t>
+          <t>Streptococcus sanguinis</t>
         </is>
       </c>
     </row>
     <row r="487">
       <c r="A487" t="inlineStr">
         <is>
-          <t>B_STRPT_GRPG</t>
+          <t>B_STRPT_GRPK</t>
         </is>
       </c>
       <c r="B487" t="inlineStr">
         <is>
-          <t>B_STRPT_DYSG</t>
+          <t>B_STRPT_SLVR</t>
         </is>
       </c>
       <c r="C487" t="inlineStr">
         <is>
-          <t>Streptococcus Group G</t>
+          <t>Streptococcus Group K</t>
         </is>
       </c>
       <c r="D487" t="inlineStr">
         <is>
-          <t>Streptococcus dysgalactiae</t>
+          <t>Streptococcus salivarius</t>
         </is>
       </c>
     </row>
     <row r="488">
       <c r="A488" t="inlineStr">
         <is>
-          <t>B_STRPT_GRPG</t>
+          <t>B_STRPT_GRPK</t>
         </is>
       </c>
       <c r="B488" t="inlineStr">
         <is>
-          <t>B_STRPT_DYSG_DYSG</t>
+          <t>B_STRPT_SLVR</t>
         </is>
       </c>
       <c r="C488" t="inlineStr">
         <is>
-          <t>Streptococcus Group G</t>
+          <t>Streptococcus Group K</t>
         </is>
       </c>
       <c r="D488" t="inlineStr">
         <is>
-          <t>Streptococcus dysgalactiae dysgalactiae</t>
+          <t>Streptococcus salivarius salivarius</t>
         </is>
       </c>
     </row>
     <row r="489">
       <c r="A489" t="inlineStr">
         <is>
-          <t>B_STRPT_GRPG</t>
+          <t>B_STRPT_GRPK</t>
         </is>
       </c>
       <c r="B489" t="inlineStr">
         <is>
-          <t>B_STRPT_DYSG_EQSM</t>
+          <t>B_STRPT_THRM</t>
         </is>
       </c>
       <c r="C489" t="inlineStr">
         <is>
-          <t>Streptococcus Group G</t>
+          <t>Streptococcus Group K</t>
         </is>
       </c>
       <c r="D489" t="inlineStr">
         <is>
-          <t>Streptococcus dysgalactiae equisimilis</t>
+          <t>Streptococcus salivarius thermophilus</t>
         </is>
       </c>
     </row>
     <row r="490">
       <c r="A490" t="inlineStr">
         <is>
-          <t>B_STRPT_GRPH</t>
+          <t>B_STRPT_GRPL</t>
         </is>
       </c>
       <c r="B490" t="inlineStr">
         <is>
-          <t>B_STRPT_SNGN</t>
+          <t>B_STRPT_DYSG</t>
         </is>
       </c>
       <c r="C490" t="inlineStr">
         <is>
-          <t>Streptococcus Group H</t>
+          <t>Streptococcus Group L</t>
         </is>
       </c>
       <c r="D490" t="inlineStr">
         <is>
-          <t>Streptococcus sanguinis</t>
+          <t>Streptococcus dysgalactiae</t>
         </is>
       </c>
     </row>
     <row r="491">
       <c r="A491" t="inlineStr">
         <is>
-          <t>B_STRPT_GRPK</t>
+          <t>B_STRPT_GRPL</t>
         </is>
       </c>
       <c r="B491" t="inlineStr">
         <is>
-          <t>B_STRPT_SLVR</t>
+          <t>B_STRPT_DYSG_DYSG</t>
         </is>
       </c>
       <c r="C491" t="inlineStr">
         <is>
-          <t>Streptococcus Group K</t>
+          <t>Streptococcus Group L</t>
         </is>
       </c>
       <c r="D491" t="inlineStr">
         <is>
-          <t>Streptococcus salivarius</t>
+          <t>Streptococcus dysgalactiae dysgalactiae</t>
         </is>
       </c>
     </row>
     <row r="492">
       <c r="A492" t="inlineStr">
         <is>
-          <t>B_STRPT_GRPK</t>
+          <t>B_STRPT_GRPL</t>
         </is>
       </c>
       <c r="B492" t="inlineStr">
         <is>
-          <t>B_STRPT_SLVR</t>
+          <t>B_STRPT_DYSG_EQSM</t>
         </is>
       </c>
       <c r="C492" t="inlineStr">
         <is>
-          <t>Streptococcus Group K</t>
+          <t>Streptococcus Group L</t>
         </is>
       </c>
       <c r="D492" t="inlineStr">
         <is>
-          <t>Streptococcus salivarius salivarius</t>
+          <t>Streptococcus dysgalactiae equisimilis</t>
         </is>
       </c>
     </row>
     <row r="493">
       <c r="A493" t="inlineStr">
         <is>
-          <t>B_STRPT_GRPK</t>
+          <t>B_STRPT_VIRI</t>
         </is>
       </c>
       <c r="B493" t="inlineStr">
         <is>
-          <t>B_STRPT_THRM</t>
+          <t>B_STRPT_MILL</t>
         </is>
       </c>
       <c r="C493" t="inlineStr">
         <is>
-          <t>Streptococcus Group K</t>
+          <t>Viridans Group Streptococcus (VGS)</t>
         </is>
       </c>
       <c r="D493" t="inlineStr">
         <is>
-          <t>Streptococcus salivarius thermophilus</t>
+          <t>Milleri Group Streptococcus (MGS)</t>
         </is>
       </c>
     </row>
     <row r="494">
       <c r="A494" t="inlineStr">
         <is>
-          <t>B_STRPT_GRPL</t>
+          <t>B_STRPT_VIRI</t>
         </is>
       </c>
       <c r="B494" t="inlineStr">
         <is>
-          <t>B_STRPT_DYSG</t>
+          <t>B_STRPT_ACDM</t>
         </is>
       </c>
       <c r="C494" t="inlineStr">
         <is>
-          <t>Streptococcus Group L</t>
+          <t>Viridans Group Streptococcus (VGS)</t>
         </is>
       </c>
       <c r="D494" t="inlineStr">
         <is>
-          <t>Streptococcus dysgalactiae</t>
+          <t>Streptococcus acidominimus</t>
         </is>
       </c>
     </row>
     <row r="495">
       <c r="A495" t="inlineStr">
         <is>
-          <t>B_STRPT_GRPL</t>
+          <t>B_STRPT_VIRI</t>
         </is>
       </c>
       <c r="B495" t="inlineStr">
         <is>
-          <t>B_STRPT_DYSG_DYSG</t>
+          <t>B_STRPT_ANGN</t>
         </is>
       </c>
       <c r="C495" t="inlineStr">
         <is>
-          <t>Streptococcus Group L</t>
+          <t>Viridans Group Streptococcus (VGS)</t>
         </is>
       </c>
       <c r="D495" t="inlineStr">
         <is>
-          <t>Streptococcus dysgalactiae dysgalactiae</t>
+          <t>Streptococcus anginosus</t>
         </is>
       </c>
     </row>
     <row r="496">
       <c r="A496" t="inlineStr">
         <is>
-          <t>B_STRPT_GRPL</t>
+          <t>B_STRPT_VIRI</t>
         </is>
       </c>
       <c r="B496" t="inlineStr">
         <is>
-          <t>B_STRPT_DYSG_EQSM</t>
+          <t>B_STRPT_ANGN_ANGN</t>
         </is>
       </c>
       <c r="C496" t="inlineStr">
         <is>
-          <t>Streptococcus Group L</t>
+          <t>Viridans Group Streptococcus (VGS)</t>
         </is>
       </c>
       <c r="D496" t="inlineStr">
         <is>
-          <t>Streptococcus dysgalactiae equisimilis</t>
+          <t>Streptococcus anginosus anginosus</t>
         </is>
       </c>
     </row>
@@ -11288,7 +11288,7 @@
       </c>
       <c r="B497" t="inlineStr">
         <is>
-          <t>B_STRPT_MILL</t>
+          <t>B_STRPT_ANGN_WHLY</t>
         </is>
       </c>
       <c r="C497" t="inlineStr">
@@ -11298,7 +11298,7 @@
       </c>
       <c r="D497" t="inlineStr">
         <is>
-          <t>Milleri Group Streptococcus (MGS)</t>
+          <t>Streptococcus anginosus whileyi</t>
         </is>
       </c>
     </row>
@@ -11310,7 +11310,7 @@
       </c>
       <c r="B498" t="inlineStr">
         <is>
-          <t>B_STRPT_ACDM</t>
+          <t>B_STRPT_CNST</t>
         </is>
       </c>
       <c r="C498" t="inlineStr">
@@ -11320,7 +11320,7 @@
       </c>
       <c r="D498" t="inlineStr">
         <is>
-          <t>Streptococcus acidominimus</t>
+          <t>Streptococcus constellatus</t>
         </is>
       </c>
     </row>
@@ -11332,7 +11332,7 @@
       </c>
       <c r="B499" t="inlineStr">
         <is>
-          <t>B_STRPT_ANGN</t>
+          <t>B_STRPT_CNST_CNST</t>
         </is>
       </c>
       <c r="C499" t="inlineStr">
@@ -11342,7 +11342,7 @@
       </c>
       <c r="D499" t="inlineStr">
         <is>
-          <t>Streptococcus anginosus</t>
+          <t>Streptococcus constellatus constellatus</t>
         </is>
       </c>
     </row>
@@ -11354,7 +11354,7 @@
       </c>
       <c r="B500" t="inlineStr">
         <is>
-          <t>B_STRPT_ANGN_ANGN</t>
+          <t>B_STRPT_CNST_PHRY</t>
         </is>
       </c>
       <c r="C500" t="inlineStr">
@@ -11364,7 +11364,7 @@
       </c>
       <c r="D500" t="inlineStr">
         <is>
-          <t>Streptococcus anginosus anginosus</t>
+          <t>Streptococcus constellatus pharyngis</t>
         </is>
       </c>
     </row>
@@ -11376,7 +11376,7 @@
       </c>
       <c r="B501" t="inlineStr">
         <is>
-          <t>B_STRPT_ANGN_WHLY</t>
+          <t>B_STRPT_CNST_VBRG</t>
         </is>
       </c>
       <c r="C501" t="inlineStr">
@@ -11386,7 +11386,7 @@
       </c>
       <c r="D501" t="inlineStr">
         <is>
-          <t>Streptococcus anginosus whileyi</t>
+          <t>Streptococcus constellatus viborgensis</t>
         </is>
       </c>
     </row>
@@ -11398,7 +11398,7 @@
       </c>
       <c r="B502" t="inlineStr">
         <is>
-          <t>B_STRPT_CNST</t>
+          <t>B_STRPT_CRCT</t>
         </is>
       </c>
       <c r="C502" t="inlineStr">
@@ -11408,7 +11408,7 @@
       </c>
       <c r="D502" t="inlineStr">
         <is>
-          <t>Streptococcus constellatus</t>
+          <t>Streptococcus criceti</t>
         </is>
       </c>
     </row>
@@ -11420,7 +11420,7 @@
       </c>
       <c r="B503" t="inlineStr">
         <is>
-          <t>B_STRPT_CNST_CNST</t>
+          <t>B_STRPT_CRST</t>
         </is>
       </c>
       <c r="C503" t="inlineStr">
@@ -11430,7 +11430,7 @@
       </c>
       <c r="D503" t="inlineStr">
         <is>
-          <t>Streptococcus constellatus constellatus</t>
+          <t>Streptococcus cristatus</t>
         </is>
       </c>
     </row>
@@ -11442,7 +11442,7 @@
       </c>
       <c r="B504" t="inlineStr">
         <is>
-          <t>B_STRPT_CNST_PHRY</t>
+          <t>B_STRPT_DOWN</t>
         </is>
       </c>
       <c r="C504" t="inlineStr">
@@ -11452,7 +11452,7 @@
       </c>
       <c r="D504" t="inlineStr">
         <is>
-          <t>Streptococcus constellatus pharyngis</t>
+          <t>Streptococcus downei</t>
         </is>
       </c>
     </row>
@@ -11464,7 +11464,7 @@
       </c>
       <c r="B505" t="inlineStr">
         <is>
-          <t>B_STRPT_CNST_VBRG</t>
+          <t>B_STRPT_EQNS</t>
         </is>
       </c>
       <c r="C505" t="inlineStr">
@@ -11474,7 +11474,7 @@
       </c>
       <c r="D505" t="inlineStr">
         <is>
-          <t>Streptococcus constellatus viborgensis</t>
+          <t>Streptococcus equinus</t>
         </is>
       </c>
     </row>
@@ -11486,7 +11486,7 @@
       </c>
       <c r="B506" t="inlineStr">
         <is>
-          <t>B_STRPT_CRCT</t>
+          <t>B_STRPT_FERS</t>
         </is>
       </c>
       <c r="C506" t="inlineStr">
@@ -11496,7 +11496,7 @@
       </c>
       <c r="D506" t="inlineStr">
         <is>
-          <t>Streptococcus criceti</t>
+          <t>Streptococcus ferus</t>
         </is>
       </c>
     </row>
@@ -11508,7 +11508,7 @@
       </c>
       <c r="B507" t="inlineStr">
         <is>
-          <t>B_STRPT_CRST</t>
+          <t>B_STRPT_GRDN</t>
         </is>
       </c>
       <c r="C507" t="inlineStr">
@@ -11518,7 +11518,7 @@
       </c>
       <c r="D507" t="inlineStr">
         <is>
-          <t>Streptococcus cristatus</t>
+          <t>Streptococcus gordonii</t>
         </is>
       </c>
     </row>
@@ -11530,7 +11530,7 @@
       </c>
       <c r="B508" t="inlineStr">
         <is>
-          <t>B_STRPT_DOWN</t>
+          <t>B_STRPT_INTR</t>
         </is>
       </c>
       <c r="C508" t="inlineStr">
@@ -11540,7 +11540,7 @@
       </c>
       <c r="D508" t="inlineStr">
         <is>
-          <t>Streptococcus downei</t>
+          <t>Streptococcus intermedius</t>
         </is>
       </c>
     </row>
@@ -11552,7 +11552,7 @@
       </c>
       <c r="B509" t="inlineStr">
         <is>
-          <t>B_STRPT_EQNS</t>
+          <t>B_STRPT_MACC</t>
         </is>
       </c>
       <c r="C509" t="inlineStr">
@@ -11562,7 +11562,7 @@
       </c>
       <c r="D509" t="inlineStr">
         <is>
-          <t>Streptococcus equinus</t>
+          <t>Streptococcus macacae</t>
         </is>
       </c>
     </row>
@@ -11574,7 +11574,7 @@
       </c>
       <c r="B510" t="inlineStr">
         <is>
-          <t>B_STRPT_FERS</t>
+          <t>B_STRPT_MITS</t>
         </is>
       </c>
       <c r="C510" t="inlineStr">
@@ -11584,7 +11584,7 @@
       </c>
       <c r="D510" t="inlineStr">
         <is>
-          <t>Streptococcus ferus</t>
+          <t>Streptococcus mitis</t>
         </is>
       </c>
     </row>
@@ -11596,7 +11596,7 @@
       </c>
       <c r="B511" t="inlineStr">
         <is>
-          <t>B_STRPT_GRDN</t>
+          <t>B_STRPT_MTNS</t>
         </is>
       </c>
       <c r="C511" t="inlineStr">
@@ -11606,7 +11606,7 @@
       </c>
       <c r="D511" t="inlineStr">
         <is>
-          <t>Streptococcus gordonii</t>
+          <t>Streptococcus mutans</t>
         </is>
       </c>
     </row>
@@ -11618,7 +11618,7 @@
       </c>
       <c r="B512" t="inlineStr">
         <is>
-          <t>B_STRPT_INTR</t>
+          <t>B_STRPT_ORLS</t>
         </is>
       </c>
       <c r="C512" t="inlineStr">
@@ -11628,7 +11628,7 @@
       </c>
       <c r="D512" t="inlineStr">
         <is>
-          <t>Streptococcus intermedius</t>
+          <t>Streptococcus oralis</t>
         </is>
       </c>
     </row>
@@ -11640,7 +11640,7 @@
       </c>
       <c r="B513" t="inlineStr">
         <is>
-          <t>B_STRPT_MACC</t>
+          <t>B_STRPT_ORLS_DNTS</t>
         </is>
       </c>
       <c r="C513" t="inlineStr">
@@ -11650,7 +11650,7 @@
       </c>
       <c r="D513" t="inlineStr">
         <is>
-          <t>Streptococcus macacae</t>
+          <t>Streptococcus oralis dentisani</t>
         </is>
       </c>
     </row>
@@ -11662,7 +11662,7 @@
       </c>
       <c r="B514" t="inlineStr">
         <is>
-          <t>B_STRPT_MITS</t>
+          <t>B_STRPT_ORLS_ORLS</t>
         </is>
       </c>
       <c r="C514" t="inlineStr">
@@ -11672,7 +11672,7 @@
       </c>
       <c r="D514" t="inlineStr">
         <is>
-          <t>Streptococcus mitis</t>
+          <t>Streptococcus oralis oralis</t>
         </is>
       </c>
     </row>
@@ -11684,7 +11684,7 @@
       </c>
       <c r="B515" t="inlineStr">
         <is>
-          <t>B_STRPT_MTNS</t>
+          <t>B_STRPT_ORLS_TGRN</t>
         </is>
       </c>
       <c r="C515" t="inlineStr">
@@ -11694,7 +11694,7 @@
       </c>
       <c r="D515" t="inlineStr">
         <is>
-          <t>Streptococcus mutans</t>
+          <t>Streptococcus oralis tigurinus</t>
         </is>
       </c>
     </row>
@@ -11706,7 +11706,7 @@
       </c>
       <c r="B516" t="inlineStr">
         <is>
-          <t>B_STRPT_ORLS</t>
+          <t>B_STRPT_PRSN</t>
         </is>
       </c>
       <c r="C516" t="inlineStr">
@@ -11716,7 +11716,7 @@
       </c>
       <c r="D516" t="inlineStr">
         <is>
-          <t>Streptococcus oralis</t>
+          <t>Streptococcus parasanguinis</t>
         </is>
       </c>
     </row>
@@ -11728,7 +11728,7 @@
       </c>
       <c r="B517" t="inlineStr">
         <is>
-          <t>B_STRPT_ORLS_DNTS</t>
+          <t>B_STRPT_RATT</t>
         </is>
       </c>
       <c r="C517" t="inlineStr">
@@ -11738,7 +11738,7 @@
       </c>
       <c r="D517" t="inlineStr">
         <is>
-          <t>Streptococcus oralis dentisani</t>
+          <t>Streptococcus ratti</t>
         </is>
       </c>
     </row>
@@ -11750,7 +11750,7 @@
       </c>
       <c r="B518" t="inlineStr">
         <is>
-          <t>B_STRPT_ORLS_ORLS</t>
+          <t>B_STRPT_SLVR</t>
         </is>
       </c>
       <c r="C518" t="inlineStr">
@@ -11760,7 +11760,7 @@
       </c>
       <c r="D518" t="inlineStr">
         <is>
-          <t>Streptococcus oralis oralis</t>
+          <t>Streptococcus salivarius</t>
         </is>
       </c>
     </row>
@@ -11772,7 +11772,7 @@
       </c>
       <c r="B519" t="inlineStr">
         <is>
-          <t>B_STRPT_ORLS_TGRN</t>
+          <t>B_STRPT_SLVR</t>
         </is>
       </c>
       <c r="C519" t="inlineStr">
@@ -11782,7 +11782,7 @@
       </c>
       <c r="D519" t="inlineStr">
         <is>
-          <t>Streptococcus oralis tigurinus</t>
+          <t>Streptococcus salivarius salivarius</t>
         </is>
       </c>
     </row>
@@ -11794,7 +11794,7 @@
       </c>
       <c r="B520" t="inlineStr">
         <is>
-          <t>B_STRPT_PRSN</t>
+          <t>B_STRPT_THRM</t>
         </is>
       </c>
       <c r="C520" t="inlineStr">
@@ -11804,7 +11804,7 @@
       </c>
       <c r="D520" t="inlineStr">
         <is>
-          <t>Streptococcus parasanguinis</t>
+          <t>Streptococcus salivarius thermophilus</t>
         </is>
       </c>
     </row>
@@ -11816,7 +11816,7 @@
       </c>
       <c r="B521" t="inlineStr">
         <is>
-          <t>B_STRPT_RATT</t>
+          <t>B_STRPT_SNGN</t>
         </is>
       </c>
       <c r="C521" t="inlineStr">
@@ -11826,7 +11826,7 @@
       </c>
       <c r="D521" t="inlineStr">
         <is>
-          <t>Streptococcus ratti</t>
+          <t>Streptococcus sanguinis</t>
         </is>
       </c>
     </row>
@@ -11838,7 +11838,7 @@
       </c>
       <c r="B522" t="inlineStr">
         <is>
-          <t>B_STRPT_SLVR</t>
+          <t>B_STRPT_SBRN</t>
         </is>
       </c>
       <c r="C522" t="inlineStr">
@@ -11848,7 +11848,7 @@
       </c>
       <c r="D522" t="inlineStr">
         <is>
-          <t>Streptococcus salivarius</t>
+          <t>Streptococcus sobrinus</t>
         </is>
       </c>
     </row>
@@ -11860,7 +11860,7 @@
       </c>
       <c r="B523" t="inlineStr">
         <is>
-          <t>B_STRPT_SLVR</t>
+          <t>B_STRPT_SUIS</t>
         </is>
       </c>
       <c r="C523" t="inlineStr">
@@ -11870,7 +11870,7 @@
       </c>
       <c r="D523" t="inlineStr">
         <is>
-          <t>Streptococcus salivarius salivarius</t>
+          <t>Streptococcus suis</t>
         </is>
       </c>
     </row>
@@ -11882,7 +11882,7 @@
       </c>
       <c r="B524" t="inlineStr">
         <is>
-          <t>B_STRPT_THRM</t>
+          <t>B_STRPT_UBRS</t>
         </is>
       </c>
       <c r="C524" t="inlineStr">
@@ -11892,7 +11892,7 @@
       </c>
       <c r="D524" t="inlineStr">
         <is>
-          <t>Streptococcus salivarius thermophilus</t>
+          <t>Streptococcus uberis</t>
         </is>
       </c>
     </row>
@@ -11904,7 +11904,7 @@
       </c>
       <c r="B525" t="inlineStr">
         <is>
-          <t>B_STRPT_SNGN</t>
+          <t>B_STRPT_VSTB</t>
         </is>
       </c>
       <c r="C525" t="inlineStr">
@@ -11914,95 +11914,95 @@
       </c>
       <c r="D525" t="inlineStr">
         <is>
-          <t>Streptococcus sanguinis</t>
+          <t>Streptococcus vestibularis</t>
         </is>
       </c>
     </row>
     <row r="526">
       <c r="A526" t="inlineStr">
         <is>
-          <t>B_STRPT_VIRI</t>
+          <t>B_YERSN_PSDT-C</t>
         </is>
       </c>
       <c r="B526" t="inlineStr">
         <is>
-          <t>B_STRPT_SBRN</t>
+          <t>B_YERSN_PSTS</t>
         </is>
       </c>
       <c r="C526" t="inlineStr">
         <is>
-          <t>Viridans Group Streptococcus (VGS)</t>
+          <t>Yersinia pseudotuberculosis complex</t>
         </is>
       </c>
       <c r="D526" t="inlineStr">
         <is>
-          <t>Streptococcus sobrinus</t>
+          <t>Yersinia pestis</t>
         </is>
       </c>
     </row>
     <row r="527">
       <c r="A527" t="inlineStr">
         <is>
-          <t>B_STRPT_VIRI</t>
+          <t>B_YERSN_PSDT-C</t>
         </is>
       </c>
       <c r="B527" t="inlineStr">
         <is>
-          <t>B_STRPT_SUIS</t>
+          <t>B_YERSN_PSDT</t>
         </is>
       </c>
       <c r="C527" t="inlineStr">
         <is>
-          <t>Viridans Group Streptococcus (VGS)</t>
+          <t>Yersinia pseudotuberculosis complex</t>
         </is>
       </c>
       <c r="D527" t="inlineStr">
         <is>
-          <t>Streptococcus suis</t>
+          <t>Yersinia pseudotuberculosis</t>
         </is>
       </c>
     </row>
     <row r="528">
       <c r="A528" t="inlineStr">
         <is>
-          <t>B_STRPT_VIRI</t>
+          <t>B_YERSN_PSDT-C</t>
         </is>
       </c>
       <c r="B528" t="inlineStr">
         <is>
-          <t>B_STRPT_UBRS</t>
+          <t>B_YERSN_PSTS</t>
         </is>
       </c>
       <c r="C528" t="inlineStr">
         <is>
-          <t>Viridans Group Streptococcus (VGS)</t>
+          <t>Yersinia pseudotuberculosis complex</t>
         </is>
       </c>
       <c r="D528" t="inlineStr">
         <is>
-          <t>Streptococcus uberis</t>
+          <t>Yersinia pseudotuberculosis pestis</t>
         </is>
       </c>
     </row>
     <row r="529">
       <c r="A529" t="inlineStr">
         <is>
-          <t>B_STRPT_VIRI</t>
+          <t>B_YERSN_PSDT-C</t>
         </is>
       </c>
       <c r="B529" t="inlineStr">
         <is>
-          <t>B_STRPT_VSTB</t>
+          <t>B_YERSN_PSDT</t>
         </is>
       </c>
       <c r="C529" t="inlineStr">
         <is>
-          <t>Viridans Group Streptococcus (VGS)</t>
+          <t>Yersinia pseudotuberculosis complex</t>
         </is>
       </c>
       <c r="D529" t="inlineStr">
         <is>
-          <t>Streptococcus vestibularis</t>
+          <t>Yersinia pseudotuberculosis pseudotuberculosis</t>
         </is>
       </c>
     </row>
@@ -12014,7 +12014,7 @@
       </c>
       <c r="B530" t="inlineStr">
         <is>
-          <t>B_YERSN_PSTS</t>
+          <t>B_YERSN_SMLS</t>
         </is>
       </c>
       <c r="C530" t="inlineStr">
@@ -12024,7 +12024,7 @@
       </c>
       <c r="D530" t="inlineStr">
         <is>
-          <t>Yersinia pestis</t>
+          <t>Yersinia similis</t>
         </is>
       </c>
     </row>
@@ -12036,7 +12036,7 @@
       </c>
       <c r="B531" t="inlineStr">
         <is>
-          <t>B_YERSN_PSDT</t>
+          <t>B_YERSN_WTRS</t>
         </is>
       </c>
       <c r="C531" t="inlineStr">
@@ -12045,94 +12045,6 @@
         </is>
       </c>
       <c r="D531" t="inlineStr">
-        <is>
-          <t>Yersinia pseudotuberculosis</t>
-        </is>
-      </c>
-    </row>
-    <row r="532">
-      <c r="A532" t="inlineStr">
-        <is>
-          <t>B_YERSN_PSDT-C</t>
-        </is>
-      </c>
-      <c r="B532" t="inlineStr">
-        <is>
-          <t>B_YERSN_PSTS</t>
-        </is>
-      </c>
-      <c r="C532" t="inlineStr">
-        <is>
-          <t>Yersinia pseudotuberculosis complex</t>
-        </is>
-      </c>
-      <c r="D532" t="inlineStr">
-        <is>
-          <t>Yersinia pseudotuberculosis pestis</t>
-        </is>
-      </c>
-    </row>
-    <row r="533">
-      <c r="A533" t="inlineStr">
-        <is>
-          <t>B_YERSN_PSDT-C</t>
-        </is>
-      </c>
-      <c r="B533" t="inlineStr">
-        <is>
-          <t>B_YERSN_PSDT</t>
-        </is>
-      </c>
-      <c r="C533" t="inlineStr">
-        <is>
-          <t>Yersinia pseudotuberculosis complex</t>
-        </is>
-      </c>
-      <c r="D533" t="inlineStr">
-        <is>
-          <t>Yersinia pseudotuberculosis pseudotuberculosis</t>
-        </is>
-      </c>
-    </row>
-    <row r="534">
-      <c r="A534" t="inlineStr">
-        <is>
-          <t>B_YERSN_PSDT-C</t>
-        </is>
-      </c>
-      <c r="B534" t="inlineStr">
-        <is>
-          <t>B_YERSN_SMLS</t>
-        </is>
-      </c>
-      <c r="C534" t="inlineStr">
-        <is>
-          <t>Yersinia pseudotuberculosis complex</t>
-        </is>
-      </c>
-      <c r="D534" t="inlineStr">
-        <is>
-          <t>Yersinia similis</t>
-        </is>
-      </c>
-    </row>
-    <row r="535">
-      <c r="A535" t="inlineStr">
-        <is>
-          <t>B_YERSN_PSDT-C</t>
-        </is>
-      </c>
-      <c r="B535" t="inlineStr">
-        <is>
-          <t>B_YERSN_WTRS</t>
-        </is>
-      </c>
-      <c r="C535" t="inlineStr">
-        <is>
-          <t>Yersinia pseudotuberculosis complex</t>
-        </is>
-      </c>
-      <c r="D535" t="inlineStr">
         <is>
           <t>Yersinia wautersii</t>
         </is>

</xml_diff>